<commit_message>
fix(worksheet): drop unused period memo and target-rate inputs, fix number formats
Removes the 'period (memo)' columns and the three calculator-only input cells (target
contribution margin rate, discount rate, target market price) that no formula used,
moves the category column next to the amount, and replaces formats that rendered a
trailing dot on whole numbers. QA unchanged: all scenarios pass.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/calculator/Pricing_Input_Worksheet.xlsx
+++ b/docs/calculator/Pricing_Input_Worksheet.xlsx
@@ -19,11 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.##"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="#,##0.##"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -109,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -122,19 +121,16 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -509,12 +505,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="56" customWidth="1" min="5" max="5"/>
   </cols>
@@ -582,7 +578,7 @@
           <t>목표 소진기간 (개월)</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n"/>
+      <c r="B8" s="6" t="n"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>초도물량을 모두 판매하려는 기간</t>
@@ -608,7 +604,7 @@
           <t>부가세율 (%)</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n"/>
+      <c r="B10" s="9" t="n"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>예: 10</t>
@@ -647,22 +643,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>활동 (to-do)</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>기간 (메모)</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>총 비용 (KRW)</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -670,72 +661,62 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="6" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="6" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="6" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="6" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="6" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="6" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="6" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="6" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="6" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="6" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>만드는 총비용 합계</t>
         </is>
       </c>
-      <c r="C26" s="12">
-        <f>SUM($C$16:$C$25)</f>
+      <c r="B26" s="11">
+        <f>SUM($B$16:$B$25)</f>
         <v/>
       </c>
     </row>
@@ -758,27 +739,22 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>활동 (to-do)</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>기간 (메모)</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>금액 / 값</t>
         </is>
       </c>
-      <c r="D29" s="11" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -787,125 +763,115 @@
     <row r="30">
       <c r="A30" s="6" t="n"/>
       <c r="B30" s="6" t="n"/>
-      <c r="C30" s="13" t="n"/>
+      <c r="C30" s="6" t="n"/>
       <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
       <c r="B31" s="6" t="n"/>
-      <c r="C31" s="13" t="n"/>
+      <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
       <c r="B32" s="6" t="n"/>
-      <c r="C32" s="13" t="n"/>
+      <c r="C32" s="6" t="n"/>
       <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="n"/>
-      <c r="C33" s="13" t="n"/>
+      <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6" t="n"/>
-      <c r="C34" s="13" t="n"/>
+      <c r="C34" s="6" t="n"/>
       <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="6" t="n"/>
-      <c r="C35" s="13" t="n"/>
+      <c r="C35" s="6" t="n"/>
       <c r="D35" s="6" t="n"/>
-      <c r="E35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="6" t="n"/>
-      <c r="C36" s="13" t="n"/>
+      <c r="C36" s="6" t="n"/>
       <c r="D36" s="6" t="n"/>
-      <c r="E36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="6" t="n"/>
-      <c r="C37" s="13" t="n"/>
+      <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
-      <c r="E37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="6" t="n"/>
-      <c r="C38" s="13" t="n"/>
+      <c r="C38" s="6" t="n"/>
       <c r="D38" s="6" t="n"/>
-      <c r="E38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="6" t="n"/>
-      <c r="C39" s="13" t="n"/>
+      <c r="C39" s="6" t="n"/>
       <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>런칭 전 총액 합계</t>
         </is>
       </c>
-      <c r="C40" s="12">
-        <f>SUMIF($D$30:$D$39,"런칭 전 총액",$C$30:$C$39)</f>
+      <c r="B40" s="11">
+        <f>SUMIF($C$30:$C$39,"런칭 전 총액",$B$30:$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>판매 시 정액 (개당) 합계</t>
         </is>
       </c>
-      <c r="C41" s="14">
-        <f>SUMIF($D$30:$D$39,"판매 시 정액 (개당)",$C$30:$C$39)</f>
+      <c r="B41" s="11">
+        <f>SUMIF($C$30:$C$39,"판매 시 정액 (개당)",$B$30:$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>판매 시 정액 (주문당) 합계</t>
         </is>
       </c>
-      <c r="C42" s="14">
-        <f>SUMIF($D$30:$D$39,"판매 시 정액 (주문당)",$C$30:$C$39)</f>
+      <c r="B42" s="11">
+        <f>SUMIF($C$30:$C$39,"판매 시 정액 (주문당)",$B$30:$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="inlineStr">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>판매 시 순매출 대비 % 합계</t>
         </is>
       </c>
-      <c r="C43" s="15">
-        <f>SUMIF($D$30:$D$39,"판매 시 순매출 대비 %",$C$30:$C$39)</f>
+      <c r="B43" s="7">
+        <f>SUMIF($C$30:$C$39,"판매 시 순매출 대비 %",$B$30:$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="inlineStr">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>판매 시 지불액 대비 % 합계</t>
         </is>
       </c>
-      <c r="C44" s="15">
-        <f>SUMIF($D$30:$D$39,"판매 시 지불액 대비 %",$C$30:$C$39)</f>
+      <c r="B44" s="7">
+        <f>SUMIF($C$30:$C$39,"판매 시 지불액 대비 %",$B$30:$B$39)</f>
         <v/>
       </c>
     </row>
@@ -915,8 +881,8 @@
           <t>구분을 고르지 않은 행 수</t>
         </is>
       </c>
-      <c r="C45" s="16">
-        <f>COUNTIFS($C$30:$C$39,"&lt;&gt;",$D$30:$D$39,"")</f>
+      <c r="B45" s="12">
+        <f>COUNTIFS($B$30:$B$39,"&lt;&gt;",$C$30:$C$39,"")</f>
         <v/>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -944,19 +910,17 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="inlineStr">
+      <c r="A49" s="10" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B49" s="11" t="inlineStr"/>
-      <c r="C49" s="11" t="inlineStr">
+      <c r="B49" s="10" t="inlineStr">
         <is>
           <t>월 금액 (KRW)</t>
         </is>
       </c>
-      <c r="D49" s="11" t="inlineStr"/>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="C49" s="10" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -964,54 +928,42 @@
     </row>
     <row r="50">
       <c r="A50" s="6" t="n"/>
-      <c r="B50" s="6" t="n"/>
-      <c r="C50" s="8" t="n"/>
-      <c r="D50" s="6" t="n"/>
-      <c r="E50" s="6" t="n"/>
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n"/>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="8" t="n"/>
-      <c r="D51" s="6" t="n"/>
-      <c r="E51" s="6" t="n"/>
+      <c r="B51" s="8" t="n"/>
+      <c r="C51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n"/>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="8" t="n"/>
-      <c r="D52" s="6" t="n"/>
-      <c r="E52" s="6" t="n"/>
+      <c r="B52" s="8" t="n"/>
+      <c r="C52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n"/>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="8" t="n"/>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
+      <c r="B53" s="8" t="n"/>
+      <c r="C53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="8" t="n"/>
-      <c r="D54" s="6" t="n"/>
-      <c r="E54" s="6" t="n"/>
+      <c r="B54" s="8" t="n"/>
+      <c r="C54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="8" t="n"/>
-      <c r="D55" s="6" t="n"/>
-      <c r="E55" s="6" t="n"/>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="6" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="11" t="inlineStr">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>월 고정운영비 합계</t>
         </is>
       </c>
-      <c r="C56" s="12">
-        <f>SUM($C$50:$C$55)</f>
+      <c r="B56" s="11">
+        <f>SUM($B$50:$B$55)</f>
         <v/>
       </c>
     </row>
@@ -1034,19 +986,19 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="inlineStr">
+      <c r="A60" s="10" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B60" s="11" t="inlineStr">
+      <c r="B60" s="10" t="inlineStr">
         <is>
           <t>값</t>
         </is>
       </c>
-      <c r="C60" s="11" t="inlineStr"/>
-      <c r="D60" s="11" t="inlineStr"/>
-      <c r="E60" s="11" t="inlineStr">
+      <c r="C60" s="10" t="inlineStr"/>
+      <c r="D60" s="10" t="inlineStr"/>
+      <c r="E60" s="10" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
@@ -1074,7 +1026,7 @@
           <t>순매출 (VAT 제외 판매가)</t>
         </is>
       </c>
-      <c r="B62" s="14">
+      <c r="B62" s="11">
         <f>IF(NOT($B$61),"",IF($B$11="예",$B$9/(1+$B$10/100),$B$9))</f>
         <v/>
       </c>
@@ -1085,7 +1037,7 @@
           <t>고객 지불액 (VAT 포함)</t>
         </is>
       </c>
-      <c r="B63" s="14">
+      <c r="B63" s="11">
         <f>IF(NOT($B$61),"",IF($B$11="예",$B$9,$B$9*(1+$B$10/100)))</f>
         <v/>
       </c>
@@ -1096,8 +1048,8 @@
           <t>개당 변동비 (판매 시)</t>
         </is>
       </c>
-      <c r="B64" s="14">
-        <f>IF(NOT($B$61),"",$C$41+$C$42+$C$43/100*$B$62+$C$44/100*$B$63)</f>
+      <c r="B64" s="11">
+        <f>IF(NOT($B$61),"",$B$41+$B$42+$B$43/100*$B$62+$B$44/100*$B$63)</f>
         <v/>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -1112,7 +1064,7 @@
           <t>판매 1개당 남는 금액</t>
         </is>
       </c>
-      <c r="B65" s="14">
+      <c r="B65" s="11">
         <f>IF(NOT($B$61),"",$B$62-$B$64)</f>
         <v/>
       </c>
@@ -1128,8 +1080,8 @@
           <t>초도 총비용</t>
         </is>
       </c>
-      <c r="B66" s="12">
-        <f>IF(NOT($B$61),"",$C$26+$C$40)</f>
+      <c r="B66" s="11">
+        <f>IF(NOT($B$61),"",$B$26+$B$40)</f>
         <v/>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -1144,8 +1096,8 @@
           <t>회수해야 할 총액</t>
         </is>
       </c>
-      <c r="B67" s="12">
-        <f>IF(NOT($B$61),"",$B$66+$C$56*$B$8)</f>
+      <c r="B67" s="11">
+        <f>IF(NOT($B$61),"",$B$66+$B$56*$B$8)</f>
         <v/>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -1160,7 +1112,7 @@
           <t>본전에 필요한 누적 판매량</t>
         </is>
       </c>
-      <c r="B68" s="14">
+      <c r="B68" s="13">
         <f>IF(NOT($B$61),"",IF($B$65&gt;0,$B$67/$B$65,"불가 (판매 1개당 남는 금액 ≤ 0)"))</f>
         <v/>
       </c>
@@ -1176,7 +1128,7 @@
           <t>필요 판매량 ÷ 수량</t>
         </is>
       </c>
-      <c r="B69" s="17">
+      <c r="B69" s="14">
         <f>IF(NOT($B$61),"",IF(AND(ISNUMBER($B$68),$B$7&gt;0),$B$68/$B$7,""))</f>
         <v/>
       </c>
@@ -1192,7 +1144,7 @@
           <t>필요 월 판매량 (소진기간 내 본전)</t>
         </is>
       </c>
-      <c r="B70" s="14">
+      <c r="B70" s="13">
         <f>IF(NOT($B$61),"",IF(AND(ISNUMBER($B$68),$B$8&gt;0),$B$68/$B$8,""))</f>
         <v/>
       </c>
@@ -1208,7 +1160,7 @@
           <t>목표 월 판매량</t>
         </is>
       </c>
-      <c r="B71" s="14">
+      <c r="B71" s="13">
         <f>IF(NOT($B$61),"",IF($B$8&gt;0,$B$7/$B$8,""))</f>
         <v/>
       </c>
@@ -1224,7 +1176,7 @@
           <t>초도물량 전량 판매 시 손익</t>
         </is>
       </c>
-      <c r="B72" s="12">
+      <c r="B72" s="11">
         <f>IF(NOT($B$61),"",$B$7*$B$65-$B$67)</f>
         <v/>
       </c>
@@ -1240,8 +1192,8 @@
           <t>초도물량 전량 판매 시 본전 판매가</t>
         </is>
       </c>
-      <c r="B73" s="14">
-        <f>IF(NOT($B$61),"",IF((1-$C$43/100-$C$44/100*(1+$B$10/100))&lt;=0,"불가 (수수료율 합계 과다)",IF($B$11="예",(1+$B$10/100),1)*(($B$67/$B$7)+$C$41+$C$42)/(1-$C$43/100-$C$44/100*(1+$B$10/100))))</f>
+      <c r="B73" s="11">
+        <f>IF(NOT($B$61),"",IF((1-$B$43/100-$B$44/100*(1+$B$10/100))&lt;=0,"불가 (수수료율 합계 과다)",IF($B$11="예",(1+$B$10/100),1)*(($B$67/$B$7)+$B$41+$B$42)/(1-$B$43/100-$B$44/100*(1+$B$10/100))))</f>
         <v/>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -1251,12 +1203,12 @@
       </c>
     </row>
     <row r="74" ht="48" customHeight="1">
-      <c r="A74" s="11" t="inlineStr">
+      <c r="A74" s="10" t="inlineStr">
         <is>
           <t>판정</t>
         </is>
       </c>
-      <c r="B74" s="18">
+      <c r="B74" s="15">
         <f>IF(NOT($B$61),"필수 입력(판매가·부가세율·VAT 여부·수량·소진기간)을 채워 주세요",IF($B$65&lt;=0,"판매 1개당 남는 금액이 0 이하입니다 — 팔수록 손해. 가격·수수료를 다시 검토하세요",IF($B$69&gt;1,"초도물량을 전부 팔아도 본전이 안 됩니다 — 가격 인상, 비용 절감, 고정비 축소 또는 기간·물량 조정을 검토하세요","초도물량으로 본전 가능 — 소진기간 안에 누적 "&amp;TEXT($B$68,"#,##0.#")&amp;"개(월 "&amp;TEXT($B$70,"#,##0.#")&amp;"개) 이상 판매 필요, 목표는 월 "&amp;TEXT($B$71,"#,##0.#")&amp;"개")))</f>
         <v/>
       </c>
@@ -1280,29 +1232,29 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="11" t="inlineStr">
+      <c r="A78" s="10" t="inlineStr">
         <is>
           <t>실제 판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B78" s="12">
+      <c r="B78" s="11">
         <f>IF($B$9="","",$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="11" t="inlineStr">
+      <c r="A79" s="10" t="inlineStr">
         <is>
           <t>부가세율 (%)</t>
         </is>
       </c>
-      <c r="B79" s="19">
+      <c r="B79" s="16">
         <f>IF($B$10="","",$B$10)</f>
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="11" t="inlineStr">
+      <c r="A80" s="10" t="inlineStr">
         <is>
           <t>VAT 포함가 체크</t>
         </is>
@@ -1313,123 +1265,91 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="11" t="inlineStr">
+      <c r="A81" s="10" t="inlineStr">
         <is>
           <t>직접원가 (개당, 초도 완전원가)</t>
         </is>
       </c>
-      <c r="B81" s="14">
-        <f>IF(NOT($B$61),"",IF($B$7&gt;0,$C$26/$B$7,""))</f>
+      <c r="B81" s="11">
+        <f>IF(NOT($B$61),"",IF($B$7&gt;0,$B$26/$B$7,""))</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="11" t="inlineStr">
+      <c r="A82" s="10" t="inlineStr">
         <is>
           <t>변동비: 정액 (개당)</t>
         </is>
       </c>
-      <c r="B82" s="14">
-        <f>$C$41</f>
+      <c r="B82" s="11">
+        <f>$B$41</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="11" t="inlineStr">
+      <c r="A83" s="10" t="inlineStr">
         <is>
           <t>변동비: 정액 (주문당)</t>
         </is>
       </c>
-      <c r="B83" s="14">
-        <f>$C$42</f>
+      <c r="B83" s="11">
+        <f>$B$42</f>
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="11" t="inlineStr">
+      <c r="A84" s="10" t="inlineStr">
         <is>
           <t>변동비: 순매출 대비 (%)</t>
         </is>
       </c>
-      <c r="B84" s="15">
-        <f>$C$43</f>
+      <c r="B84" s="7">
+        <f>$B$43</f>
         <v/>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="11" t="inlineStr">
+      <c r="A85" s="10" t="inlineStr">
         <is>
           <t>변동비: 지불액 대비 (%)</t>
         </is>
       </c>
-      <c r="B85" s="15">
-        <f>$C$44</f>
+      <c r="B85" s="7">
+        <f>$B$44</f>
         <v/>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="11" t="inlineStr">
+      <c r="A86" s="10" t="inlineStr">
         <is>
           <t>월 고정운영비 (런칭 전 총액 상각 포함, KRW)</t>
         </is>
       </c>
-      <c r="B86" s="12">
-        <f>IF(NOT($B$61),"",IF($B$8&gt;0,$C$56+$C$40/$B$8,""))</f>
+      <c r="B86" s="11">
+        <f>IF(NOT($B$61),"",IF($B$8&gt;0,$B$56+$B$40/$B$8,""))</f>
         <v/>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="11" t="inlineStr">
+      <c r="A87" s="10" t="inlineStr">
         <is>
           <t>월 계획 판매량 (개) — 목표 월 판매량</t>
         </is>
       </c>
-      <c r="B87" s="14">
+      <c r="B87" s="13">
         <f>$B$71</f>
         <v/>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="20" t="inlineStr">
-        <is>
-          <t>목표 공헌이익률 (%)</t>
-        </is>
-      </c>
-      <c r="B88" s="10" t="n"/>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>MODE B에 사용 — 본전 확인 후 목표를 정해 입력</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="20" t="inlineStr">
-        <is>
-          <t>정가 대비 할인율 (%)</t>
-        </is>
-      </c>
-      <c r="B89" s="10" t="n"/>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>MODE B 정가 역산</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="20" t="inlineStr">
-        <is>
-          <t>목표 시장가격 (KRW)</t>
-        </is>
-      </c>
-      <c r="B90" s="8" t="n"/>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>MODE C에 사용</t>
+    <row r="88" ht="30" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>목표 공헌이익률·정가 대비 할인율·목표 시장가격은 이 시트에서 입력하지 않습니다. 위 값을 계산기에 넣은 뒤 계산기에서 정하며, 각각 MODE B(목표 가격 역산), MODE C(허용 직접원가)에서 쓰입니다.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A77:E77"/>
     <mergeCell ref="A59:E59"/>
     <mergeCell ref="A48:E48"/>
@@ -1437,6 +1357,7 @@
     <mergeCell ref="B74:E74"/>
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A88:E88"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <dataValidations count="3">
@@ -1446,7 +1367,7 @@
     <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"예,아니오"</formula1>
     </dataValidation>
-    <dataValidation sqref="D30 D31 D32 D33 D34 D35 D36 D37 D38 D39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C30 C31 C32 C33 C34 C35 C36 C37 C38 C39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"런칭 전 총액,판매 시 정액 (개당),판매 시 정액 (주문당),판매 시 순매출 대비 %,판매 시 지불액 대비 %"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1465,7 +1386,7 @@
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="56" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1521,7 +1442,7 @@
           <t>양산 시 월 목표 판매량 (개)</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n"/>
+      <c r="B7" s="17" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>본전 판매가와 판정에 사용</t>
@@ -1560,22 +1481,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>활동 (to-do)</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>기간 (메모)</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>총 비용 (KRW, 양산 수량 기준)</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -1583,51 +1499,43 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="6" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="6" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="6" t="n"/>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="6" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="6" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="6" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="6" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="6" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1635,8 +1543,8 @@
           <t>양산 시 만드는 총비용 합계</t>
         </is>
       </c>
-      <c r="B21" s="12">
-        <f>SUM($C$13:$C$20)</f>
+      <c r="B21" s="11">
+        <f>SUM($B$13:$B$20)</f>
         <v/>
       </c>
     </row>
@@ -1659,19 +1567,17 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr"/>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>총 비용 (KRW)</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr"/>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -1679,31 +1585,23 @@
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n"/>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1711,8 +1609,8 @@
           <t>새 투자 합계</t>
         </is>
       </c>
-      <c r="B30" s="12">
-        <f>SUM($C$26:$C$29)</f>
+      <c r="B30" s="11">
+        <f>SUM($B$26:$B$29)</f>
         <v/>
       </c>
     </row>
@@ -1722,7 +1620,7 @@
           <t>제품/서비스 수명주기 (개월)</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n"/>
+      <c r="B31" s="6" t="n"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
           <t>새 투자가 있으면 입력 (장치는 내용연수와 수명주기 중 짧은 쪽)</t>
@@ -1746,7 +1644,7 @@
           <t>판매 시 정액 (개당·주문당 합계, KRW)</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n"/>
+      <c r="B34" s="6" t="n"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
           <t>비우면 초도의 판매 시 정액 합계</t>
@@ -1759,7 +1657,7 @@
           <t>판매 시 순매출 대비 % 합계</t>
         </is>
       </c>
-      <c r="B35" s="9" t="n"/>
+      <c r="B35" s="6" t="n"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
           <t>비우면 초도 값</t>
@@ -1772,7 +1670,7 @@
           <t>판매 시 지불액 대비 % 합계</t>
         </is>
       </c>
-      <c r="B36" s="9" t="n"/>
+      <c r="B36" s="6" t="n"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
           <t>비우면 초도 값</t>
@@ -1811,19 +1709,19 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B41" s="11" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>값</t>
         </is>
       </c>
-      <c r="C41" s="11" t="inlineStr"/>
-      <c r="D41" s="11" t="inlineStr"/>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr"/>
+      <c r="D41" s="10" t="inlineStr"/>
+      <c r="E41" s="10" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
@@ -1835,7 +1733,7 @@
           <t>적용 판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B42" s="12">
+      <c r="B42" s="11">
         <f>IF(ISNUMBER($B$8),$B$8,IF(ISNUMBER('초도'!$B$9),'초도'!$B$9,""))</f>
         <v/>
       </c>
@@ -1867,7 +1765,7 @@
           <t>순매출 (VAT 제외 판매가)</t>
         </is>
       </c>
-      <c r="B44" s="14">
+      <c r="B44" s="11">
         <f>IF(NOT($B$43),"",IF('초도'!$B$11="예",$B$42/(1+'초도'!$B$10/100),$B$42))</f>
         <v/>
       </c>
@@ -1878,7 +1776,7 @@
           <t>고객 지불액 (VAT 포함)</t>
         </is>
       </c>
-      <c r="B45" s="14">
+      <c r="B45" s="11">
         <f>IF(NOT($B$43),"",IF('초도'!$B$11="예",$B$42,$B$42*(1+'초도'!$B$10/100)))</f>
         <v/>
       </c>
@@ -1889,7 +1787,7 @@
           <t>개당 직접원가 (양산)</t>
         </is>
       </c>
-      <c r="B46" s="14">
+      <c r="B46" s="11">
         <f>IF(NOT($B$43),"",IF($B$6&gt;0,$B$21/$B$6,"수량 &gt; 0 필요"))</f>
         <v/>
       </c>
@@ -1905,8 +1803,8 @@
           <t>적용 판매 시 정액 합계</t>
         </is>
       </c>
-      <c r="B47" s="14">
-        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$34),$B$34,'초도'!$C$41+'초도'!$C$42))</f>
+      <c r="B47" s="11">
+        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$34),$B$34,'초도'!$B$41+'초도'!$B$42))</f>
         <v/>
       </c>
     </row>
@@ -1916,8 +1814,8 @@
           <t>적용 순매출 대비 % 합계</t>
         </is>
       </c>
-      <c r="B48" s="15">
-        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$35),$B$35,'초도'!$C$43))</f>
+      <c r="B48" s="7">
+        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$35),$B$35,'초도'!$B$43))</f>
         <v/>
       </c>
     </row>
@@ -1927,8 +1825,8 @@
           <t>적용 지불액 대비 % 합계</t>
         </is>
       </c>
-      <c r="B49" s="15">
-        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$36),$B$36,'초도'!$C$44))</f>
+      <c r="B49" s="7">
+        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$36),$B$36,'초도'!$B$44))</f>
         <v/>
       </c>
     </row>
@@ -1938,7 +1836,7 @@
           <t>개당 변동비 (판매 시)</t>
         </is>
       </c>
-      <c r="B50" s="14">
+      <c r="B50" s="11">
         <f>IF(NOT($B$43),"",$B$47+$B$48/100*$B$44+$B$49/100*$B$45)</f>
         <v/>
       </c>
@@ -1949,7 +1847,7 @@
           <t>개당 공헌이익</t>
         </is>
       </c>
-      <c r="B51" s="14">
+      <c r="B51" s="11">
         <f>IF(NOT($B$43),"",IF(ISNUMBER($B$46),$B$44-$B$46-$B$50,""))</f>
         <v/>
       </c>
@@ -1965,8 +1863,8 @@
           <t>적용 월 고정운영비</t>
         </is>
       </c>
-      <c r="B52" s="12">
-        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$37),$B$37,'초도'!$C$56))</f>
+      <c r="B52" s="11">
+        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$37),$B$37,'초도'!$B$56))</f>
         <v/>
       </c>
     </row>
@@ -1976,7 +1874,7 @@
           <t>월 상각액 (새 투자)</t>
         </is>
       </c>
-      <c r="B53" s="12">
+      <c r="B53" s="11">
         <f>IF(NOT($B$43),"",IF($B$30=0,0,IF(N($B$31)&gt;0,$B$30/$B$31,"수명주기 입력 필요")))</f>
         <v/>
       </c>
@@ -1992,7 +1890,7 @@
           <t>월 고정비 (상각 포함)</t>
         </is>
       </c>
-      <c r="B54" s="12">
+      <c r="B54" s="11">
         <f>IF(NOT($B$43),"",IF(ISNUMBER($B$53),$B$52+$B$53,""))</f>
         <v/>
       </c>
@@ -2008,7 +1906,7 @@
           <t>월 손익분기 판매량</t>
         </is>
       </c>
-      <c r="B55" s="14">
+      <c r="B55" s="13">
         <f>IF(NOT($B$43),"",IF(OR(NOT(ISNUMBER($B$54)),NOT(ISNUMBER($B$51))),"",IF($B$51&gt;0,$B$54/$B$51,IF($B$54=0,"해당 없음","불가 (공헌이익 ≤ 0)"))))</f>
         <v/>
       </c>
@@ -2024,7 +1922,7 @@
           <t>월 손익분기 ÷ 월 목표 판매량</t>
         </is>
       </c>
-      <c r="B56" s="17">
+      <c r="B56" s="14">
         <f>IF(NOT($B$43),"",IF(AND(ISNUMBER($B$55),$B$7&gt;0),$B$55/$B$7,""))</f>
         <v/>
       </c>
@@ -2040,7 +1938,7 @@
           <t>월 손익 (목표 월 판매량 기준)</t>
         </is>
       </c>
-      <c r="B57" s="12">
+      <c r="B57" s="11">
         <f>IF(NOT($B$43),"",IF(AND(ISNUMBER($B$54),ISNUMBER($B$51)),$B$7*$B$51-$B$54,""))</f>
         <v/>
       </c>
@@ -2051,7 +1949,7 @@
           <t>월 목표 판매량에서 본전 판매가</t>
         </is>
       </c>
-      <c r="B58" s="14">
+      <c r="B58" s="11">
         <f>IF(NOT($B$43),"",IF(OR(NOT(ISNUMBER($B$54)),NOT(ISNUMBER($B$46))),"",IF((1-$B$48/100-$B$49/100*(1+'초도'!$B$10/100))&lt;=0,"불가 (수수료율 합계 과다)",IF('초도'!$B$11="예",(1+'초도'!$B$10/100),1)*($B$46+$B$47+$B$54/$B$7)/(1-$B$48/100-$B$49/100*(1+'초도'!$B$10/100)))))</f>
         <v/>
       </c>
@@ -2062,12 +1960,12 @@
       </c>
     </row>
     <row r="59" ht="48" customHeight="1">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="A59" s="10" t="inlineStr">
         <is>
           <t>판정</t>
         </is>
       </c>
-      <c r="B59" s="18">
+      <c r="B59" s="15">
         <f>IF(NOT($B$43),"필수 입력(양산 수량·월 목표 판매량, 판매가, 초도 탭의 부가세율·VAT 여부)을 채워 주세요",IF(NOT(ISNUMBER($B$51)),"비용 입력을 확인하세요",IF($B$51&lt;=0,"개당 공헌이익이 0 이하입니다 — 팔수록 손해. 가격·원가·수수료를 다시 검토하세요",IF(NOT(ISNUMBER($B$56)),"고정비·수명주기 입력을 확인하세요",IF($B$56&gt;1,"목표 월 판매량으로는 본전이 안 됩니다 — 월 손익분기 "&amp;TEXT($B$55,"#,##0.#")&amp;"개가 필요합니다","목표 월 판매량으로 본전 가능 — 월 "&amp;TEXT($B$55,"#,##0.#")&amp;"개 이상 판매 필요")))))</f>
         <v/>
       </c>
@@ -2091,29 +1989,29 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="11" t="inlineStr">
+      <c r="A63" s="10" t="inlineStr">
         <is>
           <t>실제 판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B63" s="12">
+      <c r="B63" s="11">
         <f>$B$42</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="11" t="inlineStr">
+      <c r="A64" s="10" t="inlineStr">
         <is>
           <t>부가세율 (%)</t>
         </is>
       </c>
-      <c r="B64" s="19">
+      <c r="B64" s="16">
         <f>IF('초도'!$B$10="","",'초도'!$B$10)</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="11" t="inlineStr">
+      <c r="A65" s="10" t="inlineStr">
         <is>
           <t>VAT 포함가 체크</t>
         </is>
@@ -2124,67 +2022,67 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="11" t="inlineStr">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t>직접원가 (개당, 양산)</t>
         </is>
       </c>
-      <c r="B66" s="14">
+      <c r="B66" s="11">
         <f>$B$46</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="11" t="inlineStr">
+      <c r="A67" s="10" t="inlineStr">
         <is>
           <t>변동비: 정액 (개당·주문당 합계)</t>
         </is>
       </c>
-      <c r="B67" s="14">
+      <c r="B67" s="11">
         <f>$B$47</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="11" t="inlineStr">
+      <c r="A68" s="10" t="inlineStr">
         <is>
           <t>변동비: 순매출 대비 (%)</t>
         </is>
       </c>
-      <c r="B68" s="15">
+      <c r="B68" s="7">
         <f>$B$48</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="11" t="inlineStr">
+      <c r="A69" s="10" t="inlineStr">
         <is>
           <t>변동비: 지불액 대비 (%)</t>
         </is>
       </c>
-      <c r="B69" s="15">
+      <c r="B69" s="7">
         <f>$B$49</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="11" t="inlineStr">
+      <c r="A70" s="10" t="inlineStr">
         <is>
           <t>월 고정운영비 (상각 포함, KRW)</t>
         </is>
       </c>
-      <c r="B70" s="12">
+      <c r="B70" s="11">
         <f>$B$54</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="11" t="inlineStr">
+      <c r="A71" s="10" t="inlineStr">
         <is>
           <t>월 계획 판매량 (개) — 월 목표 판매량</t>
         </is>
       </c>
-      <c r="B71" s="14">
+      <c r="B71" s="13">
         <f>IF(ISNUMBER($B$7),$B$7,"")</f>
         <v/>
       </c>
@@ -2241,47 +2139,47 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>초도</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>양산</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>차이 (양산 − 초도)</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="11">
         <f>'초도'!$B$9</f>
         <v/>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="11">
         <f>'양산'!$B$42</f>
         <v/>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="11">
         <f>IF(AND(ISNUMBER(B6),ISNUMBER(C6)),C6-B6,"")</f>
         <v/>
       </c>
@@ -2292,40 +2190,40 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>순매출 (VAT 제외)</t>
         </is>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="11">
         <f>'초도'!$B$62</f>
         <v/>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="11">
         <f>'양산'!$B$44</f>
         <v/>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="11">
         <f>IF(AND(ISNUMBER(B7),ISNUMBER(C7)),C7-B7,"")</f>
         <v/>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>개당 직접원가</t>
         </is>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="11">
         <f>'초도'!$B$81</f>
         <v/>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="11">
         <f>'양산'!$B$46</f>
         <v/>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="11">
         <f>IF(AND(ISNUMBER(B8),ISNUMBER(C8)),C8-B8,"")</f>
         <v/>
       </c>
@@ -2336,40 +2234,40 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>개당 변동비 (판매 시)</t>
         </is>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="11">
         <f>'초도'!$B$64</f>
         <v/>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="11">
         <f>'양산'!$B$50</f>
         <v/>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="11">
         <f>IF(AND(ISNUMBER(B9),ISNUMBER(C9)),C9-B9,"")</f>
         <v/>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>개당 공헌이익</t>
         </is>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="11">
         <f>IF(AND(ISNUMBER(B7),ISNUMBER(B8),ISNUMBER(B9)),B7-B8-B9,"")</f>
         <v/>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="11">
         <f>'양산'!$B$51</f>
         <v/>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="11">
         <f>IF(AND(ISNUMBER(B10),ISNUMBER(C10)),C10-B10,"")</f>
         <v/>
       </c>
@@ -2380,20 +2278,20 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>월 고정비 (상각 포함)</t>
         </is>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="11">
         <f>'초도'!$B$86</f>
         <v/>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="11">
         <f>'양산'!$B$54</f>
         <v/>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="11">
         <f>IF(AND(ISNUMBER(B11),ISNUMBER(C11)),C11-B11,"")</f>
         <v/>
       </c>
@@ -2404,20 +2302,20 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>월 손익분기 판매량</t>
         </is>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="13">
         <f>IF(AND(ISNUMBER(B11),ISNUMBER(B10)),IF(B10&gt;0,B11/B10,IF(B11=0,"해당 없음","불가 (공헌이익 ≤ 0)")),"")</f>
         <v/>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="13">
         <f>'양산'!$B$55</f>
         <v/>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="13">
         <f>IF(AND(ISNUMBER(B12),ISNUMBER(C12)),C12-B12,"")</f>
         <v/>
       </c>
@@ -2428,20 +2326,20 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>본전 판매가 (VAT 기준은 초도 탭과 같음)</t>
         </is>
       </c>
-      <c r="B13" s="14">
+      <c r="B13" s="11">
         <f>'초도'!$B$73</f>
         <v/>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="11">
         <f>'양산'!$B$58</f>
         <v/>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="11">
         <f>IF(AND(ISNUMBER(B13),ISNUMBER(C13)),C13-B13,"")</f>
         <v/>
       </c>
@@ -2452,13 +2350,13 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>개당 직접원가 절감률</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr"/>
-      <c r="C14" s="17">
+      <c r="C14" s="14">
         <f>IF(AND(ISNUMBER(B8),ISNUMBER(C8),B8&gt;0),1-C8/B8,"")</f>
         <v/>
       </c>
@@ -2470,12 +2368,12 @@
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>해석</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="15">
         <f>IF(NOT(AND(ISNUMBER(B10),ISNUMBER(C10))),"두 탭의 필수 입력을 채우면 비교가 표시됩니다","양산하면 개당 직접원가가 "&amp;TEXT(ABS(C14),"0%")&amp;IF(C14&gt;=0," 낮아지고"," 높아지고")&amp;", 개당 공헌이익은 "&amp;TEXT(B10,"#,##0")&amp;"원에서 "&amp;TEXT(C10,"#,##0")&amp;"원이 됩니다. 월 손익분기는 "&amp;IF(AND(ISNUMBER(B12),ISNUMBER(C12)),TEXT(B12,"#,##0.#")&amp;"개에서 "&amp;TEXT(C12,"#,##0.#")&amp;"개로 바뀝니다.","확인이 필요합니다."))</f>
         <v/>
       </c>
@@ -2503,28 +2401,28 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>입력 정리 시트 사용법</t>
         </is>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>이 시트는 웹 계산기에 넣을 값을 미리 정리하고, 처음 만드는 물량(초도)으로 본전이 되는지와 규모를 키웠을 때(양산)의 차이를 가늠해 보는 양식입니다. 입력한 내용은 이 파일(내 컴퓨터)에만 저장되며 어디로도 전송되지 않습니다. 노란 칸만 입력하고, 회색 칸은 자동 계산입니다.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>탭 구성</t>
         </is>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>· 초도: 처음 만드는 물량 기준. 만드는 활동·파는 활동의 총비용을 적고 판정을 봅니다.
 · 양산: 규모를 키워 다시 만들 때 기준. 반복 비용, 새 투자, 바뀌는 변동비·고정비를 적습니다.
@@ -2534,14 +2432,14 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>초도 탭 작성 순서</t>
         </is>
       </c>
     </row>
     <row r="6" ht="160" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>① 1. 가정: 업종, 초도생산 수량(서비스는 소진기간 동안 받을 수 있는 고객 수), 목표 소진기간(개월), 판매가, 부가세, VAT 포함 여부를 입력합니다.
 ② 2. 만드는 활동: 런칭 직전까지 만드는 데 드는 일(to-do)을 한 줄씩 적고 그 일에 드는 총비용을 적습니다. 구분은 필요 없습니다. 제조는 재료·가공·금형·장치·포장, 서비스는 기획·개발·디자인 인건비 등입니다.
@@ -2552,14 +2450,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>판매 시 비용을 적는 법</t>
         </is>
       </c>
     </row>
     <row r="8" ht="112" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>· 판매 시 정액(개당/주문당): 팔 때마다 붙는 고정 금액(배송비 등). 총액이 아니라 1개 또는 1주문당 금액을 적습니다.
 · 판매 시 순매출 대비 %: VAT를 뺀 판매가의 몇 %가 붙는 비용(플랫폼 수수료 등). 퍼센트 숫자만 적습니다(예: 10).
@@ -2569,14 +2467,14 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>양산 탭 작성 순서</t>
         </is>
       </c>
     </row>
     <row r="10" ht="128" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>① 양산 수량(한 번에 만드는 수량)과 양산 시 월 목표 판매량을 입력합니다.
 ② 같은 설비를 이미 갖고 있다고 보고, 양산 수량을 다시 만들 때 또 드는 비용의 총비용을 적습니다. 초도 때 산 금형·장치는 다시 적지 않습니다.
@@ -2587,14 +2485,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>판정 읽는 법</t>
         </is>
       </c>
     </row>
     <row r="12" ht="144" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>· 초도 판정: 초도 총비용과 소진기간 동안의 월 고정운영비를 합한 '회수해야 할 총액'을, 판매 1개당 남는 금액(순매출 − 개당 변동비)으로 나눈 것이 본전에 필요한 누적 판매량입니다. 이 수량이 초도수량의 100%를 넘으면 초도물량을 모두 팔아도 본전이 안 됩니다.
 · 본전 판매가: 초도물량을 소진기간 안에 모두 팔았을 때 손익이 0이 되는 가격입니다(입력한 VAT 기준).
@@ -2604,14 +2502,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>계산기에 옮길 때 주의</t>
         </is>
       </c>
     </row>
     <row r="14" ht="80" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>· 초도 탭의 '직접원가(개당)'는 초도 총비용으로 환산한 초도 완전원가라 양산 때보다 높습니다. 지금 당장의 생존 판단에는 초도 값을, 규모를 키운 뒤의 가격 판단에는 양산 값을 쓰세요.
 · 계산기는 개당 직접원가와 월 고정비로 계산하므로 이 시트의 판정과 결과가 근사치로만 같습니다.
@@ -2620,14 +2518,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>작은 예시 (가상의 숫자)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="96" customHeight="1">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>초도 200개, 소진기간 6개월, 판매가 35,000원(VAT 포함 10%), 만드는 총비용 900만 원, 결제수수료 2.5%(판매 시 지불액 대비 %), 월 고정운영비 30만 원이면 → 회수해야 할 총액 1,080만 원, 판매 1개당 남는 금액 약 30,943원이라 본전에 약 349개가 필요합니다. 초도 200개를 모두 팔아도 본전이 안 된다는 판정이 나옵니다. 양산 탭에서 1,000개를 다시 만드는 반복 비용이 총 1,500만 원(개당 15,000원)이라면 개당 직접원가가 초도 45,000원에서 15,000원으로 줄어드는 것을 비교 탭에서 볼 수 있습니다.</t>
         </is>

</xml_diff>

<commit_message>
feat(worksheet): use a single sales unit as the basis for every amount
Adds a sales-unit input, merges per-unit and per-order fixed selling costs into one
per-sales-unit kind, renames unit wording throughout, and uses a conditional number format
so amounts show thousands separators. QA updated; all scenarios pass.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/calculator/Pricing_Input_Worksheet.xlsx
+++ b/docs/calculator/Pricing_Input_Worksheet.xlsx
@@ -19,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="[&gt;=1000]#,##0;General"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -108,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,14 +124,15 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -505,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -561,108 +563,116 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7">
-        <f>IF($B$6="서비스","소진 기간 동안 받을 수 있는 고객 수 (명)","초도생산 수량 (개)")</f>
-        <v/>
-      </c>
-      <c r="B7" s="8" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>판매 단위 (예: 낱개 1개, 6개입 세트, 1건)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>제조: 초도생산 수량. 서비스: 소진기간 동안 받을 수 있는 고객(수용) 수</t>
+          <t>판매가·수량·비용 모두 이 단위를 기준으로 적습니다. 한 번에 한 가지 판매 단위만 정리하세요</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>목표 소진기간 (개월)</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n"/>
+      <c r="A8" s="7">
+        <f>IF($B$6="서비스","소진기간 동안 받을 수 있는 고객 수","초도생산 수량")&amp;" (판매 단위 수"&amp;IF($B$7&lt;&gt;""," · 1단위 = "&amp;$B$7,"")&amp;")"</f>
+        <v/>
+      </c>
+      <c r="B8" s="8" t="n"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>초도물량을 모두 판매하려는 기간</t>
+          <t>제조: 초도생산 수량. 서비스: 소진기간 동안 받을 수 있는 고객(수용) 수 (판매 단위 수)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>실제 판매가 (KRW)</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="n"/>
+          <t>목표 소진기간 (개월)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>고객이 실제로 내는 가격</t>
+          <t>초도물량을 모두 판매하려는 기간</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>부가세율 (%)</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="n"/>
+          <t>실제 판매가 (KRW)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>예: 10</t>
+          <t>고객이 실제로 내는 가격</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>부가세율 (%)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>예: 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
           <t>위 판매가는 VAT 포함가인가?</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="B12" s="6" t="n"/>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>예 / 아니오</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>2. 만드는 활동 / How to make — 런칭 직전까지</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>초도물량을 만드는 데 드는 일(to-do)을 한 줄씩 적고, 그 일에 드는 총비용을 적으세요. 제조: 재료·가공·금형·장치·포장 등 / 서비스: 기획·개발·디자인 인건비 등. 구분 없이 총액만 적습니다.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>활동 (to-do)</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>총 비용 (KRW)</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
@@ -710,146 +720,140 @@
       <c r="C25" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>만드는 총비용 합계</t>
         </is>
       </c>
-      <c r="B26" s="11">
-        <f>SUM($B$16:$B$25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="B27" s="11">
+        <f>SUM($B$17:$B$26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>3. 파는 활동 / How to sell — 런칭 전 준비와 판매 시 비용</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>'런칭 전 총액'은 입점·샘플·초기 마케팅처럼 팔기 전에 쓰는 총비용입니다. '판매 시 …'는 팔 때마다 붙는 비용만 적습니다 (수수료·결제수수료·배송비·건당 광고비). 정액은 총액이 아니라 1개(또는 1주문)당 금액, %는 퍼센트 숫자(예: 10)로 적으세요.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>'런칭 전 총액'은 입점·샘플·초기 마케팅처럼 팔기 전에 쓰는 총비용입니다. '판매 시 …'는 팔 때마다 붙는 비용만 적습니다 (수수료·결제수수료·배송비·건당 광고비). 정액은 총액이 아니라 판매 단위 1개당 금액(판매 단위가 주문 1건이면 주문당 택배비도 여기), %는 퍼센트 숫자(예: 10)로 적으세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>활동 (to-do)</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>금액 / 값</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="D29" s="10" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6" t="n"/>
+      <c r="B31" s="12" t="n"/>
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6" t="n"/>
+      <c r="B32" s="12" t="n"/>
       <c r="C32" s="6" t="n"/>
       <c r="D32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
-      <c r="B33" s="6" t="n"/>
+      <c r="B33" s="12" t="n"/>
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
-      <c r="B34" s="6" t="n"/>
+      <c r="B34" s="12" t="n"/>
       <c r="C34" s="6" t="n"/>
       <c r="D34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
-      <c r="B35" s="6" t="n"/>
+      <c r="B35" s="12" t="n"/>
       <c r="C35" s="6" t="n"/>
       <c r="D35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
-      <c r="B36" s="6" t="n"/>
+      <c r="B36" s="12" t="n"/>
       <c r="C36" s="6" t="n"/>
       <c r="D36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
-      <c r="B37" s="6" t="n"/>
+      <c r="B37" s="12" t="n"/>
       <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
-      <c r="B38" s="6" t="n"/>
+      <c r="B38" s="12" t="n"/>
       <c r="C38" s="6" t="n"/>
       <c r="D38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
-      <c r="B39" s="6" t="n"/>
+      <c r="B39" s="12" t="n"/>
       <c r="C39" s="6" t="n"/>
       <c r="D39" s="6" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>런칭 전 총액 합계</t>
-        </is>
-      </c>
-      <c r="B40" s="11">
-        <f>SUMIF($C$30:$C$39,"런칭 전 총액",$B$30:$B$39)</f>
-        <v/>
-      </c>
+      <c r="A40" s="6" t="n"/>
+      <c r="B40" s="12" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>판매 시 정액 (개당) 합계</t>
+          <t>런칭 전 총액 합계</t>
         </is>
       </c>
       <c r="B41" s="11">
-        <f>SUMIF($C$30:$C$39,"판매 시 정액 (개당)",$B$30:$B$39)</f>
+        <f>SUMIF($C$31:$C$40,"런칭 전 총액",$B$31:$B$40)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>판매 시 정액 (주문당) 합계</t>
+          <t>판매 시 정액 (판매 단위당) 합계</t>
         </is>
       </c>
       <c r="B42" s="11">
-        <f>SUMIF($C$30:$C$39,"판매 시 정액 (주문당)",$B$30:$B$39)</f>
+        <f>SUMIF($C$31:$C$40,"판매 시 정액 (판매 단위당)",$B$31:$B$40)</f>
         <v/>
       </c>
     </row>
@@ -860,7 +864,7 @@
         </is>
       </c>
       <c r="B43" s="7">
-        <f>SUMIF($C$30:$C$39,"판매 시 순매출 대비 %",$B$30:$B$39)</f>
+        <f>SUMIF($C$31:$C$40,"판매 시 순매출 대비 %",$B$31:$B$40)</f>
         <v/>
       </c>
     </row>
@@ -871,7 +875,7 @@
         </is>
       </c>
       <c r="B44" s="7">
-        <f>SUMIF($C$30:$C$39,"판매 시 지불액 대비 %",$B$30:$B$39)</f>
+        <f>SUMIF($C$31:$C$40,"판매 시 지불액 대비 %",$B$31:$B$40)</f>
         <v/>
       </c>
     </row>
@@ -881,8 +885,8 @@
           <t>구분을 고르지 않은 행 수</t>
         </is>
       </c>
-      <c r="B45" s="12">
-        <f>COUNTIFS($B$30:$B$39,"&lt;&gt;",$C$30:$C$39,"")</f>
+      <c r="B45" s="13">
+        <f>COUNTIFS($B$31:$B$40,"&lt;&gt;",$C$31:$C$40,"")</f>
         <v/>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1011,7 +1015,7 @@
         </is>
       </c>
       <c r="B61" s="7">
-        <f>AND(ISNUMBER($B$9),ISNUMBER($B$10),OR($B$11="예",$B$11="아니오"),ISNUMBER($B$7),ISNUMBER($B$8))</f>
+        <f>AND(ISNUMBER($B$10),ISNUMBER($B$11),OR($B$12="예",$B$12="아니오"),ISNUMBER($B$8),ISNUMBER($B$9))</f>
         <v/>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -1027,7 +1031,7 @@
         </is>
       </c>
       <c r="B62" s="11">
-        <f>IF(NOT($B$61),"",IF($B$11="예",$B$9/(1+$B$10/100),$B$9))</f>
+        <f>IF(NOT($B$61),"",IF($B$12="예",$B$10/(1+$B$11/100),$B$10))</f>
         <v/>
       </c>
     </row>
@@ -1038,18 +1042,18 @@
         </is>
       </c>
       <c r="B63" s="11">
-        <f>IF(NOT($B$61),"",IF($B$11="예",$B$9,$B$9*(1+$B$10/100)))</f>
+        <f>IF(NOT($B$61),"",IF($B$12="예",$B$10,$B$10*(1+$B$11/100)))</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>개당 변동비 (판매 시)</t>
+          <t>판매 단위당 변동비 (판매 시)</t>
         </is>
       </c>
       <c r="B64" s="11">
-        <f>IF(NOT($B$61),"",$B$41+$B$42+$B$43/100*$B$62+$B$44/100*$B$63)</f>
+        <f>IF(NOT($B$61),"",$B$42+$B$43/100*$B$62+$B$44/100*$B$63)</f>
         <v/>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -1061,7 +1065,7 @@
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>판매 1개당 남는 금액</t>
+          <t>판매 단위당 남는 금액</t>
         </is>
       </c>
       <c r="B65" s="11">
@@ -1070,7 +1074,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>순매출 − 개당 변동비 (제작비·고정비 회수 전)</t>
+          <t>순매출 − 판매 단위당 변동비 (제작비·고정비 회수 전)</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1085,7 @@
         </is>
       </c>
       <c r="B66" s="11">
-        <f>IF(NOT($B$61),"",$B$26+$B$40)</f>
+        <f>IF(NOT($B$61),"",$B$27+$B$41)</f>
         <v/>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -1097,7 +1101,7 @@
         </is>
       </c>
       <c r="B67" s="11">
-        <f>IF(NOT($B$61),"",$B$66+$B$56*$B$8)</f>
+        <f>IF(NOT($B$61),"",$B$66+$B$56*$B$9)</f>
         <v/>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -1112,13 +1116,13 @@
           <t>본전에 필요한 누적 판매량</t>
         </is>
       </c>
-      <c r="B68" s="13">
-        <f>IF(NOT($B$61),"",IF($B$65&gt;0,$B$67/$B$65,"불가 (판매 1개당 남는 금액 ≤ 0)"))</f>
+      <c r="B68" s="14">
+        <f>IF(NOT($B$61),"",IF($B$65&gt;0,$B$67/$B$65,"불가 (판매 단위당 남는 금액 ≤ 0)"))</f>
         <v/>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>회수해야 할 총액 ÷ 판매 1개당 남는 금액</t>
+          <t>회수해야 할 총액 ÷ 판매 단위당 남는 금액</t>
         </is>
       </c>
     </row>
@@ -1128,8 +1132,8 @@
           <t>필요 판매량 ÷ 수량</t>
         </is>
       </c>
-      <c r="B69" s="14">
-        <f>IF(NOT($B$61),"",IF(AND(ISNUMBER($B$68),$B$7&gt;0),$B$68/$B$7,""))</f>
+      <c r="B69" s="15">
+        <f>IF(NOT($B$61),"",IF(AND(ISNUMBER($B$68),$B$8&gt;0),$B$68/$B$8,""))</f>
         <v/>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -1144,8 +1148,8 @@
           <t>필요 월 판매량 (소진기간 내 본전)</t>
         </is>
       </c>
-      <c r="B70" s="13">
-        <f>IF(NOT($B$61),"",IF(AND(ISNUMBER($B$68),$B$8&gt;0),$B$68/$B$8,""))</f>
+      <c r="B70" s="14">
+        <f>IF(NOT($B$61),"",IF(AND(ISNUMBER($B$68),$B$9&gt;0),$B$68/$B$9,""))</f>
         <v/>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -1160,8 +1164,8 @@
           <t>목표 월 판매량</t>
         </is>
       </c>
-      <c r="B71" s="13">
-        <f>IF(NOT($B$61),"",IF($B$8&gt;0,$B$7/$B$8,""))</f>
+      <c r="B71" s="14">
+        <f>IF(NOT($B$61),"",IF($B$9&gt;0,$B$8/$B$9,""))</f>
         <v/>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -1177,12 +1181,12 @@
         </is>
       </c>
       <c r="B72" s="11">
-        <f>IF(NOT($B$61),"",$B$7*$B$65-$B$67)</f>
+        <f>IF(NOT($B$61),"",$B$8*$B$65-$B$67)</f>
         <v/>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>수량 × 판매 1개당 남는 금액 − 회수해야 할 총액</t>
+          <t>수량 × 판매 단위당 남는 금액 − 회수해야 할 총액</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1197,7 @@
         </is>
       </c>
       <c r="B73" s="11">
-        <f>IF(NOT($B$61),"",IF((1-$B$43/100-$B$44/100*(1+$B$10/100))&lt;=0,"불가 (수수료율 합계 과다)",IF($B$11="예",(1+$B$10/100),1)*(($B$67/$B$7)+$B$41+$B$42)/(1-$B$43/100-$B$44/100*(1+$B$10/100))))</f>
+        <f>IF(NOT($B$61),"",IF((1-$B$43/100-$B$44/100*(1+$B$11/100))&lt;=0,"불가 (수수료율 합계 과다)",IF($B$12="예",(1+$B$11/100),1)*(($B$67/$B$8)+$B$42)/(1-$B$43/100-$B$44/100*(1+$B$11/100))))</f>
         <v/>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -1208,8 +1212,8 @@
           <t>판정</t>
         </is>
       </c>
-      <c r="B74" s="15">
-        <f>IF(NOT($B$61),"필수 입력(판매가·부가세율·VAT 여부·수량·소진기간)을 채워 주세요",IF($B$65&lt;=0,"판매 1개당 남는 금액이 0 이하입니다 — 팔수록 손해. 가격·수수료를 다시 검토하세요",IF($B$69&gt;1,"초도물량을 전부 팔아도 본전이 안 됩니다 — 가격 인상, 비용 절감, 고정비 축소 또는 기간·물량 조정을 검토하세요","초도물량으로 본전 가능 — 소진기간 안에 누적 "&amp;TEXT($B$68,"#,##0.#")&amp;"개(월 "&amp;TEXT($B$70,"#,##0.#")&amp;"개) 이상 판매 필요, 목표는 월 "&amp;TEXT($B$71,"#,##0.#")&amp;"개")))</f>
+      <c r="B74" s="16">
+        <f>IF(NOT($B$61),"필수 입력(판매가·부가세율·VAT 여부·수량·소진기간)을 채워 주세요",IF($B$65&lt;=0,"판매 단위당 남는 금액이 0 이하입니다 — 팔수록 손해. 가격·수수료를 다시 검토하세요",IF($B$69&gt;1,"초도물량을 전부 팔아도 본전이 안 됩니다 — 가격 인상, 비용 절감, 고정비 축소 또는 기간·물량 조정을 검토하세요","초도물량으로 본전 가능 — 소진기간 안에 누적 "&amp;TEXT($B$68,"#,##0.#")&amp;"단위(월 "&amp;TEXT($B$70,"#,##0.#")&amp;"단위) 이상 판매 필요, 목표는 월 "&amp;TEXT($B$71,"#,##0.#")&amp;"단위")))</f>
         <v/>
       </c>
     </row>
@@ -1224,10 +1228,10 @@
       <c r="D76" s="4" t="n"/>
       <c r="E76" s="4" t="n"/>
     </row>
-    <row r="77" ht="30" customHeight="1">
+    <row r="77" ht="45" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>웹 계산기의 같은 이름 칸에 옮겨 적으세요. 개당 직접원가는 초도 총비용으로 환산한 '초도 완전원가'라 양산 때보다 높게 나옵니다. 월 고정운영비에는 런칭 전 총액을 소진기간으로 나눈 월 상각이 포함됩니다 (계산기 결과는 이 시트의 판정과 근사치로만 같습니다).</t>
+          <t>웹 계산기의 같은 이름 칸에 옮겨 적으세요. 판매 단위당 직접원가는 초도 총비용으로 환산한 '초도 완전원가'라 양산 때보다 높게 나옵니다. 월 고정운영비에는 런칭 전 총액을 소진기간으로 나눈 월 상각이 포함됩니다 (계산기 결과는 이 시트의 판정과 근사치로만 같습니다).</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1242,7 @@
         </is>
       </c>
       <c r="B78" s="11">
-        <f>IF($B$9="","",$B$9)</f>
+        <f>IF($B$10="","",$B$10)</f>
         <v/>
       </c>
     </row>
@@ -1248,8 +1252,8 @@
           <t>부가세율 (%)</t>
         </is>
       </c>
-      <c r="B79" s="16">
-        <f>IF($B$10="","",$B$10)</f>
+      <c r="B79" s="17">
+        <f>IF($B$11="","",$B$11)</f>
         <v/>
       </c>
     </row>
@@ -1260,89 +1264,78 @@
         </is>
       </c>
       <c r="B80" s="7">
-        <f>IF($B$11="","",IF($B$11="예","체크","해제"))</f>
+        <f>IF($B$12="","",IF($B$12="예","체크","해제"))</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>직접원가 (개당, 초도 완전원가)</t>
+          <t>직접원가 (판매 단위당, 초도 완전원가)</t>
         </is>
       </c>
       <c r="B81" s="11">
-        <f>IF(NOT($B$61),"",IF($B$7&gt;0,$B$26/$B$7,""))</f>
+        <f>IF(NOT($B$61),"",IF($B$8&gt;0,$B$27/$B$8,""))</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>변동비: 정액 (개당)</t>
+          <t>변동비: 정액 (판매 단위당)</t>
         </is>
       </c>
       <c r="B82" s="11">
-        <f>$B$41</f>
+        <f>$B$42</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>변동비: 정액 (주문당)</t>
-        </is>
-      </c>
-      <c r="B83" s="11">
-        <f>$B$42</f>
+          <t>변동비: 순매출 대비 (%)</t>
+        </is>
+      </c>
+      <c r="B83" s="7">
+        <f>$B$43</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>변동비: 순매출 대비 (%)</t>
+          <t>변동비: 지불액 대비 (%)</t>
         </is>
       </c>
       <c r="B84" s="7">
-        <f>$B$43</f>
+        <f>$B$44</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>변동비: 지불액 대비 (%)</t>
-        </is>
-      </c>
-      <c r="B85" s="7">
-        <f>$B$44</f>
+          <t>월 고정운영비 (런칭 전 총액 상각 포함, KRW)</t>
+        </is>
+      </c>
+      <c r="B85" s="11">
+        <f>IF(NOT($B$61),"",IF($B$9&gt;0,$B$56+$B$41/$B$9,""))</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>월 고정운영비 (런칭 전 총액 상각 포함, KRW)</t>
-        </is>
-      </c>
-      <c r="B86" s="11">
-        <f>IF(NOT($B$61),"",IF($B$8&gt;0,$B$56+$B$40/$B$8,""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="10" t="inlineStr">
-        <is>
-          <t>월 계획 판매량 (개) — 목표 월 판매량</t>
-        </is>
-      </c>
-      <c r="B87" s="13">
+          <t>월 계획 판매량 (판매 단위 수) — 목표 월 판매량</t>
+        </is>
+      </c>
+      <c r="B86" s="14">
         <f>$B$71</f>
         <v/>
       </c>
     </row>
-    <row r="88" ht="30" customHeight="1">
-      <c r="A88" s="2" t="inlineStr">
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>목표 공헌이익률·정가 대비 할인율·목표 시장가격은 이 시트에서 입력하지 않습니다. 위 값을 계산기에 넣은 뒤 계산기에서 정하며, 각각 MODE B(목표 가격 역산), MODE C(허용 직접원가)에서 쓰입니다.</t>
         </is>
@@ -1351,24 +1344,24 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A77:E77"/>
+    <mergeCell ref="A29:E29"/>
     <mergeCell ref="A59:E59"/>
     <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A87:E87"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="B74:E74"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A88:E88"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"제조,서비스"</formula1>
     </dataValidation>
-    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"예,아니오"</formula1>
     </dataValidation>
-    <dataValidation sqref="C30 C31 C32 C33 C34 C35 C36 C37 C38 C39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"런칭 전 총액,판매 시 정액 (개당),판매 시 정액 (주문당),판매 시 순매출 대비 %,판매 시 지불액 대비 %"</formula1>
+    <dataValidation sqref="C31 C32 C33 C34 C35 C36 C37 C38 C39 C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"런칭 전 총액,판매 시 정액 (판매 단위당),판매 시 순매출 대비 %,판매 시 지불액 대비 %"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1426,7 +1419,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>양산 수량 (한 번에 만드는 수량, 개)</t>
+          <t>양산 수량 (한 번에 만드는 수량, 판매 단위 수)</t>
         </is>
       </c>
       <c r="B6" s="8" t="n"/>
@@ -1439,10 +1432,10 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>양산 시 월 목표 판매량 (개)</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="n"/>
+          <t>양산 시 월 목표 판매량 (판매 단위 수)</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>본전 판매가와 판정에 사용</t>
@@ -1641,10 +1634,10 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>판매 시 정액 (개당·주문당 합계, KRW)</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="n"/>
+          <t>판매 시 정액 (판매 단위당 합계, KRW)</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="n"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
           <t>비우면 초도의 판매 시 정액 합계</t>
@@ -1734,7 +1727,7 @@
         </is>
       </c>
       <c r="B42" s="11">
-        <f>IF(ISNUMBER($B$8),$B$8,IF(ISNUMBER('초도'!$B$9),'초도'!$B$9,""))</f>
+        <f>IF(ISNUMBER($B$8),$B$8,IF(ISNUMBER('초도'!$B$10),'초도'!$B$10,""))</f>
         <v/>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -1750,7 +1743,7 @@
         </is>
       </c>
       <c r="B43" s="7">
-        <f>AND(ISNUMBER($B$42),ISNUMBER('초도'!$B$10),OR('초도'!$B$11="예",'초도'!$B$11="아니오"),ISNUMBER($B$6),ISNUMBER($B$7))</f>
+        <f>AND(ISNUMBER($B$42),ISNUMBER('초도'!$B$11),OR('초도'!$B$12="예",'초도'!$B$12="아니오"),ISNUMBER($B$6),ISNUMBER($B$7))</f>
         <v/>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -1766,7 +1759,7 @@
         </is>
       </c>
       <c r="B44" s="11">
-        <f>IF(NOT($B$43),"",IF('초도'!$B$11="예",$B$42/(1+'초도'!$B$10/100),$B$42))</f>
+        <f>IF(NOT($B$43),"",IF('초도'!$B$12="예",$B$42/(1+'초도'!$B$11/100),$B$42))</f>
         <v/>
       </c>
     </row>
@@ -1777,14 +1770,14 @@
         </is>
       </c>
       <c r="B45" s="11">
-        <f>IF(NOT($B$43),"",IF('초도'!$B$11="예",$B$42,$B$42*(1+'초도'!$B$10/100)))</f>
+        <f>IF(NOT($B$43),"",IF('초도'!$B$12="예",$B$42,$B$42*(1+'초도'!$B$11/100)))</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>개당 직접원가 (양산)</t>
+          <t>판매 단위당 직접원가 (양산)</t>
         </is>
       </c>
       <c r="B46" s="11">
@@ -1804,7 +1797,7 @@
         </is>
       </c>
       <c r="B47" s="11">
-        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$34),$B$34,'초도'!$B$41+'초도'!$B$42))</f>
+        <f>IF(NOT($B$43),"",IF(ISNUMBER($B$34),$B$34,'초도'!$B$42))</f>
         <v/>
       </c>
     </row>
@@ -1833,7 +1826,7 @@
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>개당 변동비 (판매 시)</t>
+          <t>판매 단위당 변동비 (판매 시)</t>
         </is>
       </c>
       <c r="B50" s="11">
@@ -1844,7 +1837,7 @@
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>개당 공헌이익</t>
+          <t>판매 단위당 공헌이익</t>
         </is>
       </c>
       <c r="B51" s="11">
@@ -1853,7 +1846,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>순매출 − 개당 직접원가 − 개당 변동비</t>
+          <t>순매출 − 판매 단위당 직접원가 − 판매 단위당 변동비</t>
         </is>
       </c>
     </row>
@@ -1906,13 +1899,13 @@
           <t>월 손익분기 판매량</t>
         </is>
       </c>
-      <c r="B55" s="13">
+      <c r="B55" s="14">
         <f>IF(NOT($B$43),"",IF(OR(NOT(ISNUMBER($B$54)),NOT(ISNUMBER($B$51))),"",IF($B$51&gt;0,$B$54/$B$51,IF($B$54=0,"해당 없음","불가 (공헌이익 ≤ 0)"))))</f>
         <v/>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>월 고정비 ÷ 개당 공헌이익 (계산기 BEP와 같은 식)</t>
+          <t>월 고정비 ÷ 판매 단위당 공헌이익 (계산기 BEP와 같은 식)</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1915,7 @@
           <t>월 손익분기 ÷ 월 목표 판매량</t>
         </is>
       </c>
-      <c r="B56" s="14">
+      <c r="B56" s="15">
         <f>IF(NOT($B$43),"",IF(AND(ISNUMBER($B$55),$B$7&gt;0),$B$55/$B$7,""))</f>
         <v/>
       </c>
@@ -1950,7 +1943,7 @@
         </is>
       </c>
       <c r="B58" s="11">
-        <f>IF(NOT($B$43),"",IF(OR(NOT(ISNUMBER($B$54)),NOT(ISNUMBER($B$46))),"",IF((1-$B$48/100-$B$49/100*(1+'초도'!$B$10/100))&lt;=0,"불가 (수수료율 합계 과다)",IF('초도'!$B$11="예",(1+'초도'!$B$10/100),1)*($B$46+$B$47+$B$54/$B$7)/(1-$B$48/100-$B$49/100*(1+'초도'!$B$10/100)))))</f>
+        <f>IF(NOT($B$43),"",IF(OR(NOT(ISNUMBER($B$54)),NOT(ISNUMBER($B$46))),"",IF((1-$B$48/100-$B$49/100*(1+'초도'!$B$11/100))&lt;=0,"불가 (수수료율 합계 과다)",IF('초도'!$B$12="예",(1+'초도'!$B$11/100),1)*($B$46+$B$47+$B$54/$B$7)/(1-$B$48/100-$B$49/100*(1+'초도'!$B$11/100)))))</f>
         <v/>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -1965,8 +1958,8 @@
           <t>판정</t>
         </is>
       </c>
-      <c r="B59" s="15">
-        <f>IF(NOT($B$43),"필수 입력(양산 수량·월 목표 판매량, 판매가, 초도 탭의 부가세율·VAT 여부)을 채워 주세요",IF(NOT(ISNUMBER($B$51)),"비용 입력을 확인하세요",IF($B$51&lt;=0,"개당 공헌이익이 0 이하입니다 — 팔수록 손해. 가격·원가·수수료를 다시 검토하세요",IF(NOT(ISNUMBER($B$56)),"고정비·수명주기 입력을 확인하세요",IF($B$56&gt;1,"목표 월 판매량으로는 본전이 안 됩니다 — 월 손익분기 "&amp;TEXT($B$55,"#,##0.#")&amp;"개가 필요합니다","목표 월 판매량으로 본전 가능 — 월 "&amp;TEXT($B$55,"#,##0.#")&amp;"개 이상 판매 필요")))))</f>
+      <c r="B59" s="16">
+        <f>IF(NOT($B$43),"필수 입력(양산 수량·월 목표 판매량, 판매가, 초도 탭의 부가세율·VAT 여부)을 채워 주세요",IF(NOT(ISNUMBER($B$51)),"비용 입력을 확인하세요",IF($B$51&lt;=0,"판매 단위당 공헌이익이 0 이하입니다 — 팔수록 손해. 가격·원가·수수료를 다시 검토하세요",IF(NOT(ISNUMBER($B$56)),"고정비·수명주기 입력을 확인하세요",IF($B$56&gt;1,"목표 월 판매량으로는 본전이 안 됩니다 — 월 손익분기 "&amp;TEXT($B$55,"#,##0.#")&amp;"단위가 필요합니다","목표 월 판매량으로 본전 가능 — 월 "&amp;TEXT($B$55,"#,##0.#")&amp;"단위 이상 판매 필요")))))</f>
         <v/>
       </c>
     </row>
@@ -2005,8 +1998,8 @@
           <t>부가세율 (%)</t>
         </is>
       </c>
-      <c r="B64" s="16">
-        <f>IF('초도'!$B$10="","",'초도'!$B$10)</f>
+      <c r="B64" s="17">
+        <f>IF('초도'!$B$11="","",'초도'!$B$11)</f>
         <v/>
       </c>
     </row>
@@ -2017,14 +2010,14 @@
         </is>
       </c>
       <c r="B65" s="7">
-        <f>IF('초도'!$B$11="","",IF('초도'!$B$11="예","체크","해제"))</f>
+        <f>IF('초도'!$B$12="","",IF('초도'!$B$12="예","체크","해제"))</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>직접원가 (개당, 양산)</t>
+          <t>직접원가 (판매 단위당, 양산)</t>
         </is>
       </c>
       <c r="B66" s="11">
@@ -2035,7 +2028,7 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>변동비: 정액 (개당·주문당 합계)</t>
+          <t>변동비: 정액 (판매 단위당)</t>
         </is>
       </c>
       <c r="B67" s="11">
@@ -2079,10 +2072,10 @@
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>월 계획 판매량 (개) — 월 목표 판매량</t>
-        </is>
-      </c>
-      <c r="B71" s="13">
+          <t>월 계획 판매량 (판매 단위 수) — 월 목표 판매량</t>
+        </is>
+      </c>
+      <c r="B71" s="14">
         <f>IF(ISNUMBER($B$7),$B$7,"")</f>
         <v/>
       </c>
@@ -2134,7 +2127,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>월 손익분기는 계산기의 BEP와 같은 식(월 고정비 ÷ 개당 공헌이익)으로 양쪽을 맞췄습니다. 초도 쪽 직접원가는 초도 총비용으로 환산한 '초도 완전원가'입니다.</t>
+          <t>월 손익분기는 계산기의 BEP와 같은 식(월 고정비 ÷ 판매 단위당 공헌이익)으로 양쪽을 맞췄습니다. 초도 쪽 직접원가는 초도 총비용으로 환산한 '초도 완전원가'입니다.</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2165,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>'초도'!$B$9</f>
+        <f>'초도'!$B$10</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -2212,7 +2205,7 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>개당 직접원가</t>
+          <t>판매 단위당 직접원가</t>
         </is>
       </c>
       <c r="B8" s="11">
@@ -2236,7 +2229,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>개당 변동비 (판매 시)</t>
+          <t>판매 단위당 변동비 (판매 시)</t>
         </is>
       </c>
       <c r="B9" s="11">
@@ -2256,7 +2249,7 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>개당 공헌이익</t>
+          <t>판매 단위당 공헌이익</t>
         </is>
       </c>
       <c r="B10" s="11">
@@ -2273,7 +2266,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>순매출 − 개당 직접원가 − 개당 변동비</t>
+          <t>순매출 − 판매 단위당 직접원가 − 판매 단위당 변동비</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2277,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>'초도'!$B$86</f>
+        <f>'초도'!$B$85</f>
         <v/>
       </c>
       <c r="C11" s="11">
@@ -2307,21 +2300,21 @@
           <t>월 손익분기 판매량</t>
         </is>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="14">
         <f>IF(AND(ISNUMBER(B11),ISNUMBER(B10)),IF(B10&gt;0,B11/B10,IF(B11=0,"해당 없음","불가 (공헌이익 ≤ 0)")),"")</f>
         <v/>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="14">
         <f>'양산'!$B$55</f>
         <v/>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="14">
         <f>IF(AND(ISNUMBER(B12),ISNUMBER(C12)),C12-B12,"")</f>
         <v/>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>월 고정비 ÷ 개당 공헌이익</t>
+          <t>월 고정비 ÷ 판매 단위당 공헌이익</t>
         </is>
       </c>
     </row>
@@ -2352,18 +2345,18 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>개당 직접원가 절감률</t>
+          <t>판매 단위당 직접원가 절감률</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr"/>
-      <c r="C14" s="14">
+      <c r="C14" s="15">
         <f>IF(AND(ISNUMBER(B8),ISNUMBER(C8),B8&gt;0),1-C8/B8,"")</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>양산 시 개당 직접원가가 초도 대비 얼마나 줄었는지</t>
+          <t>양산 시 판매 단위당 직접원가가 초도 대비 얼마나 줄었는지</t>
         </is>
       </c>
     </row>
@@ -2373,8 +2366,8 @@
           <t>해석</t>
         </is>
       </c>
-      <c r="B16" s="15">
-        <f>IF(NOT(AND(ISNUMBER(B10),ISNUMBER(C10))),"두 탭의 필수 입력을 채우면 비교가 표시됩니다","양산하면 개당 직접원가가 "&amp;TEXT(ABS(C14),"0%")&amp;IF(C14&gt;=0," 낮아지고"," 높아지고")&amp;", 개당 공헌이익은 "&amp;TEXT(B10,"#,##0")&amp;"원에서 "&amp;TEXT(C10,"#,##0")&amp;"원이 됩니다. 월 손익분기는 "&amp;IF(AND(ISNUMBER(B12),ISNUMBER(C12)),TEXT(B12,"#,##0.#")&amp;"개에서 "&amp;TEXT(C12,"#,##0.#")&amp;"개로 바뀝니다.","확인이 필요합니다."))</f>
+      <c r="B16" s="16">
+        <f>IF(NOT(AND(ISNUMBER(B10),ISNUMBER(C10))),"두 탭의 필수 입력을 채우면 비교가 표시됩니다","양산하면 판매 단위당 직접원가가 "&amp;TEXT(ABS(C14),"0%")&amp;IF(C14&gt;=0," 낮아지고"," 높아지고")&amp;", 판매 단위당 공헌이익은 "&amp;TEXT(B10,"#,##0")&amp;"원에서 "&amp;TEXT(C10,"#,##0")&amp;"원이 됩니다. 월 손익분기는 "&amp;IF(AND(ISNUMBER(B12),ISNUMBER(C12)),TEXT(B12,"#,##0.#")&amp;"단위에서 "&amp;TEXT(C12,"#,##0.#")&amp;"단위로 바뀝니다.","확인이 필요합니다."))</f>
         <v/>
       </c>
     </row>
@@ -2394,35 +2387,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>입력 정리 시트 사용법</t>
         </is>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>이 시트는 웹 계산기에 넣을 값을 미리 정리하고, 처음 만드는 물량(초도)으로 본전이 되는지와 규모를 키웠을 때(양산)의 차이를 가늠해 보는 양식입니다. 입력한 내용은 이 파일(내 컴퓨터)에만 저장되며 어디로도 전송되지 않습니다. 노란 칸만 입력하고, 회색 칸은 자동 계산입니다.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>탭 구성</t>
         </is>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>· 초도: 처음 만드는 물량 기준. 만드는 활동·파는 활동의 총비용을 적고 판정을 봅니다.
 · 양산: 규모를 키워 다시 만들 때 기준. 반복 비용, 새 투자, 바뀌는 변동비·고정비를 적습니다.
@@ -2432,16 +2425,16 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>초도 탭 작성 순서</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="160" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>① 1. 가정: 업종, 초도생산 수량(서비스는 소진기간 동안 받을 수 있는 고객 수), 목표 소진기간(개월), 판매가, 부가세, VAT 포함 여부를 입력합니다.
+    <row r="6" ht="176" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>① 1. 가정: 업종, 판매 단위(낱개 1개, 6개입 세트, 1건처럼 한 번 팔 때의 단위. 판매가·수량·모든 비용이 이 단위 기준입니다), 초도생산 수량(판매 단위 수, 서비스는 소진기간 동안 받을 수 있는 고객 수), 목표 소진기간(개월), 판매가, 부가세, VAT 포함 여부를 입력합니다.
 ② 2. 만드는 활동: 런칭 직전까지 만드는 데 드는 일(to-do)을 한 줄씩 적고 그 일에 드는 총비용을 적습니다. 구분은 필요 없습니다. 제조는 재료·가공·금형·장치·포장, 서비스는 기획·개발·디자인 인건비 등입니다.
 ③ 3. 파는 활동: 런칭 전에 쓰는 총비용은 '런칭 전 총액'으로, 팔 때마다 붙는 비용은 '판매 시 …'로 구분을 고릅니다. 구분을 고르지 않은 행은 합계에서 빠지며, 표 아래 '구분을 고르지 않은 행 수'가 0이 아니면 선택하라는 뜻입니다.
 ④ 3-2. 월 고정운영비: 물량과 무관하게 매달 나가는 비용을 적습니다.
@@ -2450,31 +2443,45 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>판매 단위</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="64" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>이 시트는 판매 품목 하나, 판매 단위 하나를 기준으로 정리합니다. 판매 단위가 낱개 1개이면 모든 금액이 낱개당, 6개입 세트이면 세트당, 주문 1건이면 주문당입니다. 단위가 다르면 환산해서 적으세요(낱개 원가 1,000원인 6개입 세트는 6,000원). 낱개와 묶음을 모두 판다면 주력 판매 단위로 한 번, 다른 단위로 한 번 따로 정리합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>판매 시 비용을 적는 법</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="112" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>· 판매 시 정액(개당/주문당): 팔 때마다 붙는 고정 금액(배송비 등). 총액이 아니라 1개 또는 1주문당 금액을 적습니다.
+    <row r="10" ht="128" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>· 판매 시 정액(판매 단위당): 판매 단위 1개를 팔 때마다 붙는 고정 금액(배송비 등). 총액이 아니라 판매 단위 1개당 금액을 적습니다. 판매 단위가 주문 1건이면 주문당 택배비가 그대로 해당합니다.
 · 판매 시 순매출 대비 %: VAT를 뺀 판매가의 몇 %가 붙는 비용(플랫폼 수수료 등). 퍼센트 숫자만 적습니다(예: 10).
 · 판매 시 지불액 대비 %: VAT를 포함한 고객 결제액의 몇 %가 붙는 비용(결제수수료 등).
 제작 관련 비용은 2번에, 판매·배송 비용은 3번에만 적으세요. 같은 비용을 두 곳에 넣으면 두 번 차감됩니다.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>양산 탭 작성 순서</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="128" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
+    <row r="12" ht="128" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>① 양산 수량(한 번에 만드는 수량)과 양산 시 월 목표 판매량을 입력합니다.
 ② 같은 설비를 이미 갖고 있다고 보고, 양산 수량을 다시 만들 때 또 드는 비용의 총비용을 적습니다. 초도 때 산 금형·장치는 다시 적지 않습니다.
@@ -2484,50 +2491,50 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>판정 읽는 법</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="144" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>· 초도 판정: 초도 총비용과 소진기간 동안의 월 고정운영비를 합한 '회수해야 할 총액'을, 판매 1개당 남는 금액(순매출 − 개당 변동비)으로 나눈 것이 본전에 필요한 누적 판매량입니다. 이 수량이 초도수량의 100%를 넘으면 초도물량을 모두 팔아도 본전이 안 됩니다.
+    <row r="14" ht="144" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>· 초도 판정: 초도 총비용과 소진기간 동안의 월 고정운영비를 합한 '회수해야 할 총액'을, 판매 단위당 남는 금액(순매출 − 판매 단위당 변동비)으로 나눈 것이 본전에 필요한 누적 판매량입니다. 이 수량이 초도수량의 100%를 넘으면 초도물량을 모두 팔아도 본전이 안 됩니다.
 · 본전 판매가: 초도물량을 소진기간 안에 모두 팔았을 때 손익이 0이 되는 가격입니다(입력한 VAT 기준).
-· 양산 판정: 개당 공헌이익(순매출 − 개당 직접원가 − 개당 변동비), 월 손익분기 판매량(월 고정비 ÷ 개당 공헌이익), 월 목표 판매량과의 비교를 봅니다.
-· 비교 탭: 개당 직접원가 절감률, 개당 공헌이익, 월 손익분기가 초도에서 양산으로 어떻게 바뀌는지 봅니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+· 양산 판정: 판매 단위당 공헌이익(순매출 − 판매 단위당 직접원가 − 판매 단위당 변동비), 월 손익분기 판매량(월 고정비 ÷ 판매 단위당 공헌이익), 월 목표 판매량과의 비교를 봅니다.
+· 비교 탭: 판매 단위당 직접원가 절감률, 판매 단위당 공헌이익, 월 손익분기가 초도에서 양산으로 어떻게 바뀌는지 봅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>계산기에 옮길 때 주의</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="80" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>· 초도 탭의 '직접원가(개당)'는 초도 총비용으로 환산한 초도 완전원가라 양산 때보다 높습니다. 지금 당장의 생존 판단에는 초도 값을, 규모를 키운 뒤의 가격 판단에는 양산 값을 쓰세요.
-· 계산기는 개당 직접원가와 월 고정비로 계산하므로 이 시트의 판정과 결과가 근사치로만 같습니다.
+    <row r="16" ht="96" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>· 초도 탭의 '직접원가(판매 단위당)'는 초도 총비용으로 환산한 초도 완전원가라 양산 때보다 높습니다. 지금 당장의 생존 판단에는 초도 값을, 규모를 키운 뒤의 가격 판단에는 양산 값을 쓰세요.
+· 계산기는 판매 단위당 직접원가와 월 고정비로 계산하므로 이 시트의 판정과 결과가 근사치로만 같습니다.
 · 판정은 재고·외상 같은 시차와 추가 생산을 반영하지 않는 간이 판단이며, 세법상 감가상각과 다를 수 있는 가격 판단용 관리 계산입니다.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>작은 예시 (가상의 숫자)</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="96" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>초도 200개, 소진기간 6개월, 판매가 35,000원(VAT 포함 10%), 만드는 총비용 900만 원, 결제수수료 2.5%(판매 시 지불액 대비 %), 월 고정운영비 30만 원이면 → 회수해야 할 총액 1,080만 원, 판매 1개당 남는 금액 약 30,943원이라 본전에 약 349개가 필요합니다. 초도 200개를 모두 팔아도 본전이 안 된다는 판정이 나옵니다. 양산 탭에서 1,000개를 다시 만드는 반복 비용이 총 1,500만 원(개당 15,000원)이라면 개당 직접원가가 초도 45,000원에서 15,000원으로 줄어드는 것을 비교 탭에서 볼 수 있습니다.</t>
+    <row r="18" ht="112" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>초도 200개(판매 단위: 낱개 1개), 소진기간 6개월, 판매가 35,000원(VAT 포함 10%), 만드는 총비용 900만 원, 결제수수료 2.5%(판매 시 지불액 대비 %), 월 고정운영비 30만 원이면 → 회수해야 할 총액 1,080만 원, 판매 단위당 남는 금액 약 30,943원이라 본전에 약 349개가 필요합니다. 초도 200개를 모두 팔아도 본전이 안 된다는 판정이 나옵니다. 양산 탭에서 1,000개를 다시 만드는 반복 비용이 총 1,500만 원(판매 단위당 15,000원)이라면 판매 단위당 직접원가가 초도 45,000원에서 15,000원으로 줄어드는 것을 비교 탭에서 볼 수 있습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(worksheet): wrap assumption labels and relabel quantity/period for services
The long quantity label spilled over the input cell and looked auto-filled. Labels now wrap,
and for services the quantity is a target sales count (not a capacity) and the period a
target sales period. Formulas unchanged; QA passes.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/calculator/Pricing_Input_Worksheet.xlsx
+++ b/docs/calculator/Pricing_Input_Worksheet.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -119,12 +119,18 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -558,12 +564,12 @@
       <c r="B6" s="6" t="n"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>제조 또는 서비스 (아래 수량 항목의 이름이 바뀝니다)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+          <t>제조 또는 서비스 (아래 수량·기간 항목의 이름이 바뀝니다)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>판매 단위 (예: 낱개 1개, 6개입 세트, 1건)</t>
         </is>
@@ -575,28 +581,27 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="7">
-        <f>IF($B$6="서비스","소진기간 동안 받을 수 있는 고객 수","초도생산 수량")&amp;" (판매 단위 수"&amp;IF($B$7&lt;&gt;""," · 1단위 = "&amp;$B$7,"")&amp;")"</f>
-        <v/>
-      </c>
-      <c r="B8" s="8" t="n"/>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="8">
+        <f>IF($B$6="서비스","목표 판매 수","초도생산 수량")&amp;" (판매 단위 수"&amp;IF($B$7&lt;&gt;""," · 1단위 = "&amp;$B$7,"")&amp;")"</f>
+        <v/>
+      </c>
+      <c r="B8" s="9" t="n"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>제조: 초도생산 수량. 서비스: 소진기간 동안 받을 수 있는 고객(수용) 수 (판매 단위 수)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>목표 소진기간 (개월)</t>
-        </is>
+          <t>제조: 초도생산 수량 (판매 단위 수). 서비스: 이 기간 안에 팔려는 목표 판매 수 — 수용 한도가 아니라 목표로 적으세요</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="8">
+        <f>IF($B$6="서비스","목표 판매 기간 (개월)","목표 소진기간 (개월)")</f>
+        <v/>
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>초도물량을 모두 판매하려는 기간</t>
+          <t>초도물량(서비스는 목표 판매 수)을 모두 판매하려는 기간</t>
         </is>
       </c>
     </row>
@@ -606,7 +611,7 @@
           <t>실제 판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n"/>
+      <c r="B10" s="9" t="n"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>고객이 실제로 내는 가격</t>
@@ -619,7 +624,7 @@
           <t>부가세율 (%)</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n"/>
+      <c r="B11" s="10" t="n"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>예: 10</t>
@@ -658,17 +663,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>활동 (to-do)</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>총 비용 (KRW)</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -676,61 +681,61 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
-      <c r="B17" s="8" t="n"/>
+      <c r="B17" s="9" t="n"/>
       <c r="C17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
-      <c r="B18" s="8" t="n"/>
+      <c r="B18" s="9" t="n"/>
       <c r="C18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
-      <c r="B19" s="8" t="n"/>
+      <c r="B19" s="9" t="n"/>
       <c r="C19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
-      <c r="B20" s="8" t="n"/>
+      <c r="B20" s="9" t="n"/>
       <c r="C20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
-      <c r="B21" s="8" t="n"/>
+      <c r="B21" s="9" t="n"/>
       <c r="C21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
-      <c r="B22" s="8" t="n"/>
+      <c r="B22" s="9" t="n"/>
       <c r="C22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
-      <c r="B23" s="8" t="n"/>
+      <c r="B23" s="9" t="n"/>
       <c r="C23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
-      <c r="B24" s="8" t="n"/>
+      <c r="B24" s="9" t="n"/>
       <c r="C24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
-      <c r="B25" s="8" t="n"/>
+      <c r="B25" s="9" t="n"/>
       <c r="C25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
-      <c r="B26" s="8" t="n"/>
+      <c r="B26" s="9" t="n"/>
       <c r="C26" s="6" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>만드는 총비용 합계</t>
         </is>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="12">
         <f>SUM($B$17:$B$26)</f>
         <v/>
       </c>
@@ -754,22 +759,22 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>활동 (to-do)</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>금액 / 값</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -777,115 +782,115 @@
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
-      <c r="B31" s="12" t="n"/>
+      <c r="B31" s="13" t="n"/>
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
-      <c r="B32" s="12" t="n"/>
+      <c r="B32" s="13" t="n"/>
       <c r="C32" s="6" t="n"/>
       <c r="D32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
-      <c r="B33" s="12" t="n"/>
+      <c r="B33" s="13" t="n"/>
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
-      <c r="B34" s="12" t="n"/>
+      <c r="B34" s="13" t="n"/>
       <c r="C34" s="6" t="n"/>
       <c r="D34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
-      <c r="B35" s="12" t="n"/>
+      <c r="B35" s="13" t="n"/>
       <c r="C35" s="6" t="n"/>
       <c r="D35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
-      <c r="B36" s="12" t="n"/>
+      <c r="B36" s="13" t="n"/>
       <c r="C36" s="6" t="n"/>
       <c r="D36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
-      <c r="B37" s="12" t="n"/>
+      <c r="B37" s="13" t="n"/>
       <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
-      <c r="B38" s="12" t="n"/>
+      <c r="B38" s="13" t="n"/>
       <c r="C38" s="6" t="n"/>
       <c r="D38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
-      <c r="B39" s="12" t="n"/>
+      <c r="B39" s="13" t="n"/>
       <c r="C39" s="6" t="n"/>
       <c r="D39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
-      <c r="B40" s="12" t="n"/>
+      <c r="B40" s="13" t="n"/>
       <c r="C40" s="6" t="n"/>
       <c r="D40" s="6" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>런칭 전 총액 합계</t>
         </is>
       </c>
-      <c r="B41" s="11">
+      <c r="B41" s="12">
         <f>SUMIF($C$31:$C$40,"런칭 전 총액",$B$31:$B$40)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="inlineStr">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>판매 시 정액 (판매 단위당) 합계</t>
         </is>
       </c>
-      <c r="B42" s="11">
+      <c r="B42" s="12">
         <f>SUMIF($C$31:$C$40,"판매 시 정액 (판매 단위당)",$B$31:$B$40)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>판매 시 순매출 대비 % 합계</t>
         </is>
       </c>
-      <c r="B43" s="7">
+      <c r="B43" s="14">
         <f>SUMIF($C$31:$C$40,"판매 시 순매출 대비 %",$B$31:$B$40)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t>판매 시 지불액 대비 % 합계</t>
         </is>
       </c>
-      <c r="B44" s="7">
+      <c r="B44" s="14">
         <f>SUMIF($C$31:$C$40,"판매 시 지불액 대비 %",$B$31:$B$40)</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>구분을 고르지 않은 행 수</t>
         </is>
       </c>
-      <c r="B45" s="13">
+      <c r="B45" s="15">
         <f>COUNTIFS($B$31:$B$40,"&lt;&gt;",$C$31:$C$40,"")</f>
         <v/>
       </c>
@@ -914,17 +919,17 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="inlineStr">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B49" s="10" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
         <is>
           <t>월 금액 (KRW)</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
+      <c r="C49" s="11" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -932,41 +937,41 @@
     </row>
     <row r="50">
       <c r="A50" s="6" t="n"/>
-      <c r="B50" s="8" t="n"/>
+      <c r="B50" s="9" t="n"/>
       <c r="C50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n"/>
-      <c r="B51" s="8" t="n"/>
+      <c r="B51" s="9" t="n"/>
       <c r="C51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n"/>
-      <c r="B52" s="8" t="n"/>
+      <c r="B52" s="9" t="n"/>
       <c r="C52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n"/>
-      <c r="B53" s="8" t="n"/>
+      <c r="B53" s="9" t="n"/>
       <c r="C53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>
-      <c r="B54" s="8" t="n"/>
+      <c r="B54" s="9" t="n"/>
       <c r="C54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>
-      <c r="B55" s="8" t="n"/>
+      <c r="B55" s="9" t="n"/>
       <c r="C55" s="6" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="10" t="inlineStr">
+      <c r="A56" s="11" t="inlineStr">
         <is>
           <t>월 고정운영비 합계</t>
         </is>
       </c>
-      <c r="B56" s="11">
+      <c r="B56" s="12">
         <f>SUM($B$50:$B$55)</f>
         <v/>
       </c>
@@ -990,31 +995,31 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="10" t="inlineStr">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B60" s="10" t="inlineStr">
+      <c r="B60" s="11" t="inlineStr">
         <is>
           <t>값</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr"/>
-      <c r="D60" s="10" t="inlineStr"/>
-      <c r="E60" s="10" t="inlineStr">
+      <c r="C60" s="11" t="inlineStr"/>
+      <c r="D60" s="11" t="inlineStr"/>
+      <c r="E60" s="11" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="7" t="inlineStr">
+      <c r="A61" s="14" t="inlineStr">
         <is>
           <t>필수 입력 완료</t>
         </is>
       </c>
-      <c r="B61" s="7">
+      <c r="B61" s="14">
         <f>AND(ISNUMBER($B$10),ISNUMBER($B$11),OR($B$12="예",$B$12="아니오"),ISNUMBER($B$8),ISNUMBER($B$9))</f>
         <v/>
       </c>
@@ -1025,34 +1030,34 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="7" t="inlineStr">
+      <c r="A62" s="14" t="inlineStr">
         <is>
           <t>순매출 (VAT 제외 판매가)</t>
         </is>
       </c>
-      <c r="B62" s="11">
+      <c r="B62" s="12">
         <f>IF(NOT($B$61),"",IF($B$12="예",$B$10/(1+$B$11/100),$B$10))</f>
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="7" t="inlineStr">
+      <c r="A63" s="14" t="inlineStr">
         <is>
           <t>고객 지불액 (VAT 포함)</t>
         </is>
       </c>
-      <c r="B63" s="11">
+      <c r="B63" s="12">
         <f>IF(NOT($B$61),"",IF($B$12="예",$B$10,$B$10*(1+$B$11/100)))</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="inlineStr">
+      <c r="A64" s="14" t="inlineStr">
         <is>
           <t>판매 단위당 변동비 (판매 시)</t>
         </is>
       </c>
-      <c r="B64" s="11">
+      <c r="B64" s="12">
         <f>IF(NOT($B$61),"",$B$42+$B$43/100*$B$62+$B$44/100*$B$63)</f>
         <v/>
       </c>
@@ -1063,12 +1068,12 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="7" t="inlineStr">
+      <c r="A65" s="14" t="inlineStr">
         <is>
           <t>판매 단위당 남는 금액</t>
         </is>
       </c>
-      <c r="B65" s="11">
+      <c r="B65" s="12">
         <f>IF(NOT($B$61),"",$B$62-$B$64)</f>
         <v/>
       </c>
@@ -1079,12 +1084,12 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="7" t="inlineStr">
+      <c r="A66" s="14" t="inlineStr">
         <is>
           <t>초도 총비용</t>
         </is>
       </c>
-      <c r="B66" s="11">
+      <c r="B66" s="12">
         <f>IF(NOT($B$61),"",$B$27+$B$41)</f>
         <v/>
       </c>
@@ -1095,12 +1100,12 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="7" t="inlineStr">
+      <c r="A67" s="14" t="inlineStr">
         <is>
           <t>회수해야 할 총액</t>
         </is>
       </c>
-      <c r="B67" s="11">
+      <c r="B67" s="12">
         <f>IF(NOT($B$61),"",$B$66+$B$56*$B$9)</f>
         <v/>
       </c>
@@ -1111,12 +1116,12 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="7" t="inlineStr">
+      <c r="A68" s="14" t="inlineStr">
         <is>
           <t>본전에 필요한 누적 판매량</t>
         </is>
       </c>
-      <c r="B68" s="14">
+      <c r="B68" s="16">
         <f>IF(NOT($B$61),"",IF($B$65&gt;0,$B$67/$B$65,"불가 (판매 단위당 남는 금액 ≤ 0)"))</f>
         <v/>
       </c>
@@ -1127,12 +1132,12 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="7" t="inlineStr">
+      <c r="A69" s="14" t="inlineStr">
         <is>
           <t>필요 판매량 ÷ 수량</t>
         </is>
       </c>
-      <c r="B69" s="15">
+      <c r="B69" s="17">
         <f>IF(NOT($B$61),"",IF(AND(ISNUMBER($B$68),$B$8&gt;0),$B$68/$B$8,""))</f>
         <v/>
       </c>
@@ -1143,12 +1148,12 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="7" t="inlineStr">
+      <c r="A70" s="14" t="inlineStr">
         <is>
           <t>필요 월 판매량 (소진기간 내 본전)</t>
         </is>
       </c>
-      <c r="B70" s="14">
+      <c r="B70" s="16">
         <f>IF(NOT($B$61),"",IF(AND(ISNUMBER($B$68),$B$9&gt;0),$B$68/$B$9,""))</f>
         <v/>
       </c>
@@ -1159,12 +1164,12 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="inlineStr">
+      <c r="A71" s="14" t="inlineStr">
         <is>
           <t>목표 월 판매량</t>
         </is>
       </c>
-      <c r="B71" s="14">
+      <c r="B71" s="16">
         <f>IF(NOT($B$61),"",IF($B$9&gt;0,$B$8/$B$9,""))</f>
         <v/>
       </c>
@@ -1175,12 +1180,12 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="inlineStr">
+      <c r="A72" s="14" t="inlineStr">
         <is>
           <t>초도물량 전량 판매 시 손익</t>
         </is>
       </c>
-      <c r="B72" s="11">
+      <c r="B72" s="12">
         <f>IF(NOT($B$61),"",$B$8*$B$65-$B$67)</f>
         <v/>
       </c>
@@ -1191,12 +1196,12 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="7" t="inlineStr">
+      <c r="A73" s="14" t="inlineStr">
         <is>
           <t>초도물량 전량 판매 시 본전 판매가</t>
         </is>
       </c>
-      <c r="B73" s="11">
+      <c r="B73" s="12">
         <f>IF(NOT($B$61),"",IF((1-$B$43/100-$B$44/100*(1+$B$11/100))&lt;=0,"불가 (수수료율 합계 과다)",IF($B$12="예",(1+$B$11/100),1)*(($B$67/$B$8)+$B$42)/(1-$B$43/100-$B$44/100*(1+$B$11/100))))</f>
         <v/>
       </c>
@@ -1207,12 +1212,12 @@
       </c>
     </row>
     <row r="74" ht="48" customHeight="1">
-      <c r="A74" s="10" t="inlineStr">
+      <c r="A74" s="11" t="inlineStr">
         <is>
           <t>판정</t>
         </is>
       </c>
-      <c r="B74" s="16">
+      <c r="B74" s="18">
         <f>IF(NOT($B$61),"필수 입력(판매가·부가세율·VAT 여부·수량·소진기간)을 채워 주세요",IF($B$65&lt;=0,"판매 단위당 남는 금액이 0 이하입니다 — 팔수록 손해. 가격·수수료를 다시 검토하세요",IF($B$69&gt;1,"초도물량을 전부 팔아도 본전이 안 됩니다 — 가격 인상, 비용 절감, 고정비 축소 또는 기간·물량 조정을 검토하세요","초도물량으로 본전 가능 — 소진기간 안에 누적 "&amp;TEXT($B$68,"#,##0.#")&amp;"단위(월 "&amp;TEXT($B$70,"#,##0.#")&amp;"단위) 이상 판매 필요, 목표는 월 "&amp;TEXT($B$71,"#,##0.#")&amp;"단위")))</f>
         <v/>
       </c>
@@ -1236,100 +1241,100 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="10" t="inlineStr">
+      <c r="A78" s="11" t="inlineStr">
         <is>
           <t>실제 판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B78" s="11">
+      <c r="B78" s="12">
         <f>IF($B$10="","",$B$10)</f>
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="10" t="inlineStr">
+      <c r="A79" s="11" t="inlineStr">
         <is>
           <t>부가세율 (%)</t>
         </is>
       </c>
-      <c r="B79" s="17">
+      <c r="B79" s="19">
         <f>IF($B$11="","",$B$11)</f>
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="10" t="inlineStr">
+      <c r="A80" s="11" t="inlineStr">
         <is>
           <t>VAT 포함가 체크</t>
         </is>
       </c>
-      <c r="B80" s="7">
+      <c r="B80" s="14">
         <f>IF($B$12="","",IF($B$12="예","체크","해제"))</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="10" t="inlineStr">
+      <c r="A81" s="11" t="inlineStr">
         <is>
           <t>직접원가 (판매 단위당, 초도 완전원가)</t>
         </is>
       </c>
-      <c r="B81" s="11">
+      <c r="B81" s="12">
         <f>IF(NOT($B$61),"",IF($B$8&gt;0,$B$27/$B$8,""))</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="10" t="inlineStr">
+      <c r="A82" s="11" t="inlineStr">
         <is>
           <t>변동비: 정액 (판매 단위당)</t>
         </is>
       </c>
-      <c r="B82" s="11">
+      <c r="B82" s="12">
         <f>$B$42</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="10" t="inlineStr">
+      <c r="A83" s="11" t="inlineStr">
         <is>
           <t>변동비: 순매출 대비 (%)</t>
         </is>
       </c>
-      <c r="B83" s="7">
+      <c r="B83" s="14">
         <f>$B$43</f>
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="10" t="inlineStr">
+      <c r="A84" s="11" t="inlineStr">
         <is>
           <t>변동비: 지불액 대비 (%)</t>
         </is>
       </c>
-      <c r="B84" s="7">
+      <c r="B84" s="14">
         <f>$B$44</f>
         <v/>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="10" t="inlineStr">
+      <c r="A85" s="11" t="inlineStr">
         <is>
           <t>월 고정운영비 (런칭 전 총액 상각 포함, KRW)</t>
         </is>
       </c>
-      <c r="B85" s="11">
+      <c r="B85" s="12">
         <f>IF(NOT($B$61),"",IF($B$9&gt;0,$B$56+$B$41/$B$9,""))</f>
         <v/>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="10" t="inlineStr">
+      <c r="A86" s="11" t="inlineStr">
         <is>
           <t>월 계획 판매량 (판매 단위 수) — 목표 월 판매량</t>
         </is>
       </c>
-      <c r="B86" s="14">
+      <c r="B86" s="16">
         <f>$B$71</f>
         <v/>
       </c>
@@ -1422,7 +1427,7 @@
           <t>양산 수량 (한 번에 만드는 수량, 판매 단위 수)</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n"/>
+      <c r="B6" s="9" t="n"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>이 수량을 다시 만들 때의 반복 비용을 아래 2번에 적습니다</t>
@@ -1435,7 +1440,7 @@
           <t>양산 시 월 목표 판매량 (판매 단위 수)</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>본전 판매가와 판정에 사용</t>
@@ -1448,7 +1453,7 @@
           <t>양산 시 판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
+      <c r="B8" s="9" t="n"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>비우면 초도 판매가와 같음 (초도와 같은 VAT 기준)</t>
@@ -1474,17 +1479,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>활동 (to-do)</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>총 비용 (KRW, 양산 수량 기준)</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -1492,51 +1497,51 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
-      <c r="B13" s="8" t="n"/>
+      <c r="B13" s="9" t="n"/>
       <c r="C13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
-      <c r="B14" s="8" t="n"/>
+      <c r="B14" s="9" t="n"/>
       <c r="C14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
-      <c r="B15" s="8" t="n"/>
+      <c r="B15" s="9" t="n"/>
       <c r="C15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
-      <c r="B16" s="8" t="n"/>
+      <c r="B16" s="9" t="n"/>
       <c r="C16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
-      <c r="B17" s="8" t="n"/>
+      <c r="B17" s="9" t="n"/>
       <c r="C17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
-      <c r="B18" s="8" t="n"/>
+      <c r="B18" s="9" t="n"/>
       <c r="C18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
-      <c r="B19" s="8" t="n"/>
+      <c r="B19" s="9" t="n"/>
       <c r="C19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
-      <c r="B20" s="8" t="n"/>
+      <c r="B20" s="9" t="n"/>
       <c r="C20" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>양산 시 만드는 총비용 합계</t>
         </is>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="12">
         <f>SUM($B$13:$B$20)</f>
         <v/>
       </c>
@@ -1560,17 +1565,17 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>총 비용 (KRW)</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
@@ -1578,31 +1583,31 @@
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
-      <c r="B26" s="8" t="n"/>
+      <c r="B26" s="9" t="n"/>
       <c r="C26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>
-      <c r="B27" s="8" t="n"/>
+      <c r="B27" s="9" t="n"/>
       <c r="C27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
-      <c r="B28" s="8" t="n"/>
+      <c r="B28" s="9" t="n"/>
       <c r="C28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n"/>
-      <c r="B29" s="8" t="n"/>
+      <c r="B29" s="9" t="n"/>
       <c r="C29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>새 투자 합계</t>
         </is>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="12">
         <f>SUM($B$26:$B$29)</f>
         <v/>
       </c>
@@ -1637,7 +1642,7 @@
           <t>판매 시 정액 (판매 단위당 합계, KRW)</t>
         </is>
       </c>
-      <c r="B34" s="12" t="n"/>
+      <c r="B34" s="13" t="n"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
           <t>비우면 초도의 판매 시 정액 합계</t>
@@ -1676,7 +1681,7 @@
           <t>월 고정운영비 (KRW)</t>
         </is>
       </c>
-      <c r="B37" s="8" t="n"/>
+      <c r="B37" s="9" t="n"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
           <t>비우면 초도의 월 고정운영비 합계</t>
@@ -1702,31 +1707,31 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B41" s="10" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>값</t>
         </is>
       </c>
-      <c r="C41" s="10" t="inlineStr"/>
-      <c r="D41" s="10" t="inlineStr"/>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr"/>
+      <c r="D41" s="11" t="inlineStr"/>
+      <c r="E41" s="11" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>적용 판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B42" s="11">
+      <c r="B42" s="12">
         <f>IF(ISNUMBER($B$8),$B$8,IF(ISNUMBER('초도'!$B$10),'초도'!$B$10,""))</f>
         <v/>
       </c>
@@ -1737,12 +1742,12 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>필수 입력 완료</t>
         </is>
       </c>
-      <c r="B43" s="7">
+      <c r="B43" s="14">
         <f>AND(ISNUMBER($B$42),ISNUMBER('초도'!$B$11),OR('초도'!$B$12="예",'초도'!$B$12="아니오"),ISNUMBER($B$6),ISNUMBER($B$7))</f>
         <v/>
       </c>
@@ -1753,34 +1758,34 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>순매출 (VAT 제외 판매가)</t>
         </is>
       </c>
-      <c r="B44" s="11">
+      <c r="B44" s="12">
         <f>IF(NOT($B$43),"",IF('초도'!$B$12="예",$B$42/(1+'초도'!$B$11/100),$B$42))</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>고객 지불액 (VAT 포함)</t>
         </is>
       </c>
-      <c r="B45" s="11">
+      <c r="B45" s="12">
         <f>IF(NOT($B$43),"",IF('초도'!$B$12="예",$B$42,$B$42*(1+'초도'!$B$11/100)))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>판매 단위당 직접원가 (양산)</t>
         </is>
       </c>
-      <c r="B46" s="11">
+      <c r="B46" s="12">
         <f>IF(NOT($B$43),"",IF($B$6&gt;0,$B$21/$B$6,"수량 &gt; 0 필요"))</f>
         <v/>
       </c>
@@ -1791,56 +1796,56 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>적용 판매 시 정액 합계</t>
         </is>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="12">
         <f>IF(NOT($B$43),"",IF(ISNUMBER($B$34),$B$34,'초도'!$B$42))</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
+      <c r="A48" s="14" t="inlineStr">
         <is>
           <t>적용 순매출 대비 % 합계</t>
         </is>
       </c>
-      <c r="B48" s="7">
+      <c r="B48" s="14">
         <f>IF(NOT($B$43),"",IF(ISNUMBER($B$35),$B$35,'초도'!$B$43))</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
+      <c r="A49" s="14" t="inlineStr">
         <is>
           <t>적용 지불액 대비 % 합계</t>
         </is>
       </c>
-      <c r="B49" s="7">
+      <c r="B49" s="14">
         <f>IF(NOT($B$43),"",IF(ISNUMBER($B$36),$B$36,'초도'!$B$44))</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
+      <c r="A50" s="14" t="inlineStr">
         <is>
           <t>판매 단위당 변동비 (판매 시)</t>
         </is>
       </c>
-      <c r="B50" s="11">
+      <c r="B50" s="12">
         <f>IF(NOT($B$43),"",$B$47+$B$48/100*$B$44+$B$49/100*$B$45)</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>판매 단위당 공헌이익</t>
         </is>
       </c>
-      <c r="B51" s="11">
+      <c r="B51" s="12">
         <f>IF(NOT($B$43),"",IF(ISNUMBER($B$46),$B$44-$B$46-$B$50,""))</f>
         <v/>
       </c>
@@ -1851,23 +1856,23 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t>적용 월 고정운영비</t>
         </is>
       </c>
-      <c r="B52" s="11">
+      <c r="B52" s="12">
         <f>IF(NOT($B$43),"",IF(ISNUMBER($B$37),$B$37,'초도'!$B$56))</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
+      <c r="A53" s="14" t="inlineStr">
         <is>
           <t>월 상각액 (새 투자)</t>
         </is>
       </c>
-      <c r="B53" s="11">
+      <c r="B53" s="12">
         <f>IF(NOT($B$43),"",IF($B$30=0,0,IF(N($B$31)&gt;0,$B$30/$B$31,"수명주기 입력 필요")))</f>
         <v/>
       </c>
@@ -1878,12 +1883,12 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
+      <c r="A54" s="14" t="inlineStr">
         <is>
           <t>월 고정비 (상각 포함)</t>
         </is>
       </c>
-      <c r="B54" s="11">
+      <c r="B54" s="12">
         <f>IF(NOT($B$43),"",IF(ISNUMBER($B$53),$B$52+$B$53,""))</f>
         <v/>
       </c>
@@ -1894,12 +1899,12 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
+      <c r="A55" s="14" t="inlineStr">
         <is>
           <t>월 손익분기 판매량</t>
         </is>
       </c>
-      <c r="B55" s="14">
+      <c r="B55" s="16">
         <f>IF(NOT($B$43),"",IF(OR(NOT(ISNUMBER($B$54)),NOT(ISNUMBER($B$51))),"",IF($B$51&gt;0,$B$54/$B$51,IF($B$54=0,"해당 없음","불가 (공헌이익 ≤ 0)"))))</f>
         <v/>
       </c>
@@ -1910,12 +1915,12 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="inlineStr">
+      <c r="A56" s="14" t="inlineStr">
         <is>
           <t>월 손익분기 ÷ 월 목표 판매량</t>
         </is>
       </c>
-      <c r="B56" s="15">
+      <c r="B56" s="17">
         <f>IF(NOT($B$43),"",IF(AND(ISNUMBER($B$55),$B$7&gt;0),$B$55/$B$7,""))</f>
         <v/>
       </c>
@@ -1926,23 +1931,23 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
+      <c r="A57" s="14" t="inlineStr">
         <is>
           <t>월 손익 (목표 월 판매량 기준)</t>
         </is>
       </c>
-      <c r="B57" s="11">
+      <c r="B57" s="12">
         <f>IF(NOT($B$43),"",IF(AND(ISNUMBER($B$54),ISNUMBER($B$51)),$B$7*$B$51-$B$54,""))</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>월 목표 판매량에서 본전 판매가</t>
         </is>
       </c>
-      <c r="B58" s="11">
+      <c r="B58" s="12">
         <f>IF(NOT($B$43),"",IF(OR(NOT(ISNUMBER($B$54)),NOT(ISNUMBER($B$46))),"",IF((1-$B$48/100-$B$49/100*(1+'초도'!$B$11/100))&lt;=0,"불가 (수수료율 합계 과다)",IF('초도'!$B$12="예",(1+'초도'!$B$11/100),1)*($B$46+$B$47+$B$54/$B$7)/(1-$B$48/100-$B$49/100*(1+'초도'!$B$11/100)))))</f>
         <v/>
       </c>
@@ -1953,12 +1958,12 @@
       </c>
     </row>
     <row r="59" ht="48" customHeight="1">
-      <c r="A59" s="10" t="inlineStr">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>판정</t>
         </is>
       </c>
-      <c r="B59" s="16">
+      <c r="B59" s="18">
         <f>IF(NOT($B$43),"필수 입력(양산 수량·월 목표 판매량, 판매가, 초도 탭의 부가세율·VAT 여부)을 채워 주세요",IF(NOT(ISNUMBER($B$51)),"비용 입력을 확인하세요",IF($B$51&lt;=0,"판매 단위당 공헌이익이 0 이하입니다 — 팔수록 손해. 가격·원가·수수료를 다시 검토하세요",IF(NOT(ISNUMBER($B$56)),"고정비·수명주기 입력을 확인하세요",IF($B$56&gt;1,"목표 월 판매량으로는 본전이 안 됩니다 — 월 손익분기 "&amp;TEXT($B$55,"#,##0.#")&amp;"단위가 필요합니다","목표 월 판매량으로 본전 가능 — 월 "&amp;TEXT($B$55,"#,##0.#")&amp;"단위 이상 판매 필요")))))</f>
         <v/>
       </c>
@@ -1982,100 +1987,100 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="10" t="inlineStr">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>실제 판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B63" s="11">
+      <c r="B63" s="12">
         <f>$B$42</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="10" t="inlineStr">
+      <c r="A64" s="11" t="inlineStr">
         <is>
           <t>부가세율 (%)</t>
         </is>
       </c>
-      <c r="B64" s="17">
+      <c r="B64" s="19">
         <f>IF('초도'!$B$11="","",'초도'!$B$11)</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="10" t="inlineStr">
+      <c r="A65" s="11" t="inlineStr">
         <is>
           <t>VAT 포함가 체크</t>
         </is>
       </c>
-      <c r="B65" s="7">
+      <c r="B65" s="14">
         <f>IF('초도'!$B$12="","",IF('초도'!$B$12="예","체크","해제"))</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="10" t="inlineStr">
+      <c r="A66" s="11" t="inlineStr">
         <is>
           <t>직접원가 (판매 단위당, 양산)</t>
         </is>
       </c>
-      <c r="B66" s="11">
+      <c r="B66" s="12">
         <f>$B$46</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="10" t="inlineStr">
+      <c r="A67" s="11" t="inlineStr">
         <is>
           <t>변동비: 정액 (판매 단위당)</t>
         </is>
       </c>
-      <c r="B67" s="11">
+      <c r="B67" s="12">
         <f>$B$47</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="10" t="inlineStr">
+      <c r="A68" s="11" t="inlineStr">
         <is>
           <t>변동비: 순매출 대비 (%)</t>
         </is>
       </c>
-      <c r="B68" s="7">
+      <c r="B68" s="14">
         <f>$B$48</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="10" t="inlineStr">
+      <c r="A69" s="11" t="inlineStr">
         <is>
           <t>변동비: 지불액 대비 (%)</t>
         </is>
       </c>
-      <c r="B69" s="7">
+      <c r="B69" s="14">
         <f>$B$49</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="10" t="inlineStr">
+      <c r="A70" s="11" t="inlineStr">
         <is>
           <t>월 고정운영비 (상각 포함, KRW)</t>
         </is>
       </c>
-      <c r="B70" s="11">
+      <c r="B70" s="12">
         <f>$B$54</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="10" t="inlineStr">
+      <c r="A71" s="11" t="inlineStr">
         <is>
           <t>월 계획 판매량 (판매 단위 수) — 월 목표 판매량</t>
         </is>
       </c>
-      <c r="B71" s="14">
+      <c r="B71" s="16">
         <f>IF(ISNUMBER($B$7),$B$7,"")</f>
         <v/>
       </c>
@@ -2132,47 +2137,47 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>초도</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>양산</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>차이 (양산 − 초도)</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>판매가 (KRW)</t>
         </is>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="12">
         <f>'초도'!$B$10</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="12">
         <f>'양산'!$B$42</f>
         <v/>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="12">
         <f>IF(AND(ISNUMBER(B6),ISNUMBER(C6)),C6-B6,"")</f>
         <v/>
       </c>
@@ -2183,40 +2188,40 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>순매출 (VAT 제외)</t>
         </is>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="12">
         <f>'초도'!$B$62</f>
         <v/>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="12">
         <f>'양산'!$B$44</f>
         <v/>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="12">
         <f>IF(AND(ISNUMBER(B7),ISNUMBER(C7)),C7-B7,"")</f>
         <v/>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>판매 단위당 직접원가</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="12">
         <f>'초도'!$B$81</f>
         <v/>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="12">
         <f>'양산'!$B$46</f>
         <v/>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="12">
         <f>IF(AND(ISNUMBER(B8),ISNUMBER(C8)),C8-B8,"")</f>
         <v/>
       </c>
@@ -2227,40 +2232,40 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>판매 단위당 변동비 (판매 시)</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="12">
         <f>'초도'!$B$64</f>
         <v/>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="12">
         <f>'양산'!$B$50</f>
         <v/>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="12">
         <f>IF(AND(ISNUMBER(B9),ISNUMBER(C9)),C9-B9,"")</f>
         <v/>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>판매 단위당 공헌이익</t>
         </is>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="12">
         <f>IF(AND(ISNUMBER(B7),ISNUMBER(B8),ISNUMBER(B9)),B7-B8-B9,"")</f>
         <v/>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="12">
         <f>'양산'!$B$51</f>
         <v/>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="12">
         <f>IF(AND(ISNUMBER(B10),ISNUMBER(C10)),C10-B10,"")</f>
         <v/>
       </c>
@@ -2271,20 +2276,20 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>월 고정비 (상각 포함)</t>
         </is>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="12">
         <f>'초도'!$B$85</f>
         <v/>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="12">
         <f>'양산'!$B$54</f>
         <v/>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="12">
         <f>IF(AND(ISNUMBER(B11),ISNUMBER(C11)),C11-B11,"")</f>
         <v/>
       </c>
@@ -2295,20 +2300,20 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>월 손익분기 판매량</t>
         </is>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="16">
         <f>IF(AND(ISNUMBER(B11),ISNUMBER(B10)),IF(B10&gt;0,B11/B10,IF(B11=0,"해당 없음","불가 (공헌이익 ≤ 0)")),"")</f>
         <v/>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="16">
         <f>'양산'!$B$55</f>
         <v/>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="16">
         <f>IF(AND(ISNUMBER(B12),ISNUMBER(C12)),C12-B12,"")</f>
         <v/>
       </c>
@@ -2319,20 +2324,20 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>본전 판매가 (VAT 기준은 초도 탭과 같음)</t>
         </is>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="12">
         <f>'초도'!$B$73</f>
         <v/>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="12">
         <f>'양산'!$B$58</f>
         <v/>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="12">
         <f>IF(AND(ISNUMBER(B13),ISNUMBER(C13)),C13-B13,"")</f>
         <v/>
       </c>
@@ -2343,17 +2348,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>판매 단위당 직접원가 절감률</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr"/>
-      <c r="C14" s="15">
+      <c r="B14" s="14" t="inlineStr"/>
+      <c r="C14" s="17">
         <f>IF(AND(ISNUMBER(B8),ISNUMBER(C8),B8&gt;0),1-C8/B8,"")</f>
         <v/>
       </c>
-      <c r="D14" s="7" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>양산 시 판매 단위당 직접원가가 초도 대비 얼마나 줄었는지</t>
@@ -2361,12 +2366,12 @@
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>해석</t>
         </is>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="18">
         <f>IF(NOT(AND(ISNUMBER(B10),ISNUMBER(C10))),"두 탭의 필수 입력을 채우면 비교가 표시됩니다","양산하면 판매 단위당 직접원가가 "&amp;TEXT(ABS(C14),"0%")&amp;IF(C14&gt;=0," 낮아지고"," 높아지고")&amp;", 판매 단위당 공헌이익은 "&amp;TEXT(B10,"#,##0")&amp;"원에서 "&amp;TEXT(C10,"#,##0")&amp;"원이 됩니다. 월 손익분기는 "&amp;IF(AND(ISNUMBER(B12),ISNUMBER(C12)),TEXT(B12,"#,##0.#")&amp;"단위에서 "&amp;TEXT(C12,"#,##0.#")&amp;"단위로 바뀝니다.","확인이 필요합니다."))</f>
         <v/>
       </c>
@@ -2394,28 +2399,28 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>입력 정리 시트 사용법</t>
         </is>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>이 시트는 웹 계산기에 넣을 값을 미리 정리하고, 처음 만드는 물량(초도)으로 본전이 되는지와 규모를 키웠을 때(양산)의 차이를 가늠해 보는 양식입니다. 입력한 내용은 이 파일(내 컴퓨터)에만 저장되며 어디로도 전송되지 않습니다. 노란 칸만 입력하고, 회색 칸은 자동 계산입니다.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>탭 구성</t>
         </is>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>· 초도: 처음 만드는 물량 기준. 만드는 활동·파는 활동의 총비용을 적고 판정을 봅니다.
 · 양산: 규모를 키워 다시 만들 때 기준. 반복 비용, 새 투자, 바뀌는 변동비·고정비를 적습니다.
@@ -2425,16 +2430,16 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>초도 탭 작성 순서</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="176" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
-        <is>
-          <t>① 1. 가정: 업종, 판매 단위(낱개 1개, 6개입 세트, 1건처럼 한 번 팔 때의 단위. 판매가·수량·모든 비용이 이 단위 기준입니다), 초도생산 수량(판매 단위 수, 서비스는 소진기간 동안 받을 수 있는 고객 수), 목표 소진기간(개월), 판매가, 부가세, VAT 포함 여부를 입력합니다.
+    <row r="6" ht="192" customHeight="1">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>① 1. 가정: 업종, 판매 단위(낱개 1개, 6개입 세트, 1건처럼 한 번 팔 때의 단위. 판매가·수량·모든 비용이 이 단위 기준입니다), 초도생산 수량(판매 단위 수. 서비스는 수용 한도가 아니라 이 기간 안에 팔려는 목표 판매 수), 목표 소진기간(서비스는 목표 판매 기간, 개월), 판매가, 부가세, VAT 포함 여부를 입력합니다.
 ② 2. 만드는 활동: 런칭 직전까지 만드는 데 드는 일(to-do)을 한 줄씩 적고 그 일에 드는 총비용을 적습니다. 구분은 필요 없습니다. 제조는 재료·가공·금형·장치·포장, 서비스는 기획·개발·디자인 인건비 등입니다.
 ③ 3. 파는 활동: 런칭 전에 쓰는 총비용은 '런칭 전 총액'으로, 팔 때마다 붙는 비용은 '판매 시 …'로 구분을 고릅니다. 구분을 고르지 않은 행은 합계에서 빠지며, 표 아래 '구분을 고르지 않은 행 수'가 0이 아니면 선택하라는 뜻입니다.
 ④ 3-2. 월 고정운영비: 물량과 무관하게 매달 나가는 비용을 적습니다.
@@ -2443,28 +2448,28 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>판매 단위</t>
         </is>
       </c>
     </row>
     <row r="8" ht="64" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>이 시트는 판매 품목 하나, 판매 단위 하나를 기준으로 정리합니다. 판매 단위가 낱개 1개이면 모든 금액이 낱개당, 6개입 세트이면 세트당, 주문 1건이면 주문당입니다. 단위가 다르면 환산해서 적으세요(낱개 원가 1,000원인 6개입 세트는 6,000원). 낱개와 묶음을 모두 판다면 주력 판매 단위로 한 번, 다른 단위로 한 번 따로 정리합니다.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>판매 시 비용을 적는 법</t>
         </is>
       </c>
     </row>
     <row r="10" ht="128" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>· 판매 시 정액(판매 단위당): 판매 단위 1개를 팔 때마다 붙는 고정 금액(배송비 등). 총액이 아니라 판매 단위 1개당 금액을 적습니다. 판매 단위가 주문 1건이면 주문당 택배비가 그대로 해당합니다.
 · 판매 시 순매출 대비 %: VAT를 뺀 판매가의 몇 %가 붙는 비용(플랫폼 수수료 등). 퍼센트 숫자만 적습니다(예: 10).
@@ -2474,14 +2479,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>양산 탭 작성 순서</t>
         </is>
       </c>
     </row>
     <row r="12" ht="128" customHeight="1">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>① 양산 수량(한 번에 만드는 수량)과 양산 시 월 목표 판매량을 입력합니다.
 ② 같은 설비를 이미 갖고 있다고 보고, 양산 수량을 다시 만들 때 또 드는 비용의 총비용을 적습니다. 초도 때 산 금형·장치는 다시 적지 않습니다.
@@ -2492,14 +2497,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>판정 읽는 법</t>
         </is>
       </c>
     </row>
     <row r="14" ht="144" customHeight="1">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>· 초도 판정: 초도 총비용과 소진기간 동안의 월 고정운영비를 합한 '회수해야 할 총액'을, 판매 단위당 남는 금액(순매출 − 판매 단위당 변동비)으로 나눈 것이 본전에 필요한 누적 판매량입니다. 이 수량이 초도수량의 100%를 넘으면 초도물량을 모두 팔아도 본전이 안 됩니다.
 · 본전 판매가: 초도물량을 소진기간 안에 모두 팔았을 때 손익이 0이 되는 가격입니다(입력한 VAT 기준).
@@ -2509,14 +2514,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>계산기에 옮길 때 주의</t>
         </is>
       </c>
     </row>
     <row r="16" ht="96" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>· 초도 탭의 '직접원가(판매 단위당)'는 초도 총비용으로 환산한 초도 완전원가라 양산 때보다 높습니다. 지금 당장의 생존 판단에는 초도 값을, 규모를 키운 뒤의 가격 판단에는 양산 값을 쓰세요.
 · 계산기는 판매 단위당 직접원가와 월 고정비로 계산하므로 이 시트의 판정과 결과가 근사치로만 같습니다.
@@ -2525,14 +2530,14 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>작은 예시 (가상의 숫자)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="112" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>초도 200개(판매 단위: 낱개 1개), 소진기간 6개월, 판매가 35,000원(VAT 포함 10%), 만드는 총비용 900만 원, 결제수수료 2.5%(판매 시 지불액 대비 %), 월 고정운영비 30만 원이면 → 회수해야 할 총액 1,080만 원, 판매 단위당 남는 금액 약 30,943원이라 본전에 약 349개가 필요합니다. 초도 200개를 모두 팔아도 본전이 안 된다는 판정이 나옵니다. 양산 탭에서 1,000개를 다시 만드는 반복 비용이 총 1,500만 원(판매 단위당 15,000원)이라면 판매 단위당 직접원가가 초도 45,000원에서 15,000원으로 줄어드는 것을 비교 탭에서 볼 수 있습니다.</t>
         </is>

</xml_diff>

<commit_message>
feat(calculator): paste the worksheet's calculator-values table to fill the inputs
Adds a paste box that reads the input worksheet's 'values to type into the calculator'
table in the browser (nothing is sent anywhere) and fills price, VAT, direct cost,
variable costs, fixed cost and planned volume. The worksheet notes and guide tab explain
the step, and the worksheet QA now runs the calculator's parser (node) against each
scenario's copied table.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/calculator/Pricing_Input_Worksheet.xlsx
+++ b/docs/calculator/Pricing_Input_Worksheet.xlsx
@@ -1032,7 +1032,7 @@
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>순매출 (VAT 제외 판매가)</t>
+          <t>판매 단위당 순매출 (VAT 제외 판매가)</t>
         </is>
       </c>
       <c r="B62" s="12">
@@ -1043,7 +1043,7 @@
     <row r="63">
       <c r="A63" s="14" t="inlineStr">
         <is>
-          <t>고객 지불액 (VAT 포함)</t>
+          <t>판매 단위당 고객 지불액 (VAT 포함)</t>
         </is>
       </c>
       <c r="B63" s="12">
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="B74" s="18">
-        <f>IF(NOT($B$61),"필수 입력(판매가·부가세율·VAT 여부·수량·소진기간)을 채워 주세요",IF($B$65&lt;=0,"판매 단위당 남는 금액이 0 이하입니다 — 팔수록 손해. 가격·수수료를 다시 검토하세요",IF($B$69&gt;1,"초도물량을 전부 팔아도 본전이 안 됩니다 — 가격 인상, 비용 절감, 고정비 축소 또는 기간·물량 조정을 검토하세요","초도물량으로 본전 가능 — 소진기간 안에 누적 "&amp;TEXT($B$68,"#,##0.#")&amp;"단위(월 "&amp;TEXT($B$70,"#,##0.#")&amp;"단위) 이상 판매 필요, 목표는 월 "&amp;TEXT($B$71,"#,##0.#")&amp;"단위")))</f>
+        <f>IF(NOT($B$61),"필수 입력(판매가·부가세율·VAT 여부·수량·소진기간)을 채워 주세요",IF($B$65&lt;=0,"판매 단위당 남는 금액이 0 이하입니다 — 팔수록 손해. 가격·수수료를 다시 검토하세요",IF($B$69&gt;1,"초도물량을 전부 팔아도 본전이 안 됩니다 — 가격 인상, 비용 절감, 고정비 축소 또는 기간·물량 조정을 검토하세요","초도물량으로 본전 가능 — 소진기간 안에 누적 "&amp;IF(ROUND($B$68,1)=INT(ROUND($B$68,1)),TEXT(ROUND($B$68,1),"#,##0"),TEXT(ROUND($B$68,1),"#,##0.0"))&amp;"단위(월 "&amp;IF(ROUND($B$70,1)=INT(ROUND($B$70,1)),TEXT(ROUND($B$70,1),"#,##0"),TEXT(ROUND($B$70,1),"#,##0.0"))&amp;"단위) 이상 판매 필요, 목표는 월 "&amp;IF(ROUND($B$71,1)=INT(ROUND($B$71,1)),TEXT(ROUND($B$71,1),"#,##0"),TEXT(ROUND($B$71,1),"#,##0.0"))&amp;"단위")))</f>
         <v/>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
     <row r="77" ht="45" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>웹 계산기의 같은 이름 칸에 옮겨 적으세요. 판매 단위당 직접원가는 초도 총비용으로 환산한 '초도 완전원가'라 양산 때보다 높게 나옵니다. 월 고정운영비에는 런칭 전 총액을 소진기간으로 나눈 월 상각이 포함됩니다 (계산기 결과는 이 시트의 판정과 근사치로만 같습니다).</t>
+          <t>이 표(라벨과 값 두 열)를 복사해 웹 계산기의 '시트 값 붙여넣기'에 붙여넣으면 자동으로 채워집니다. 직접 옮겨 적어도 됩니다. 판매 단위당 직접원가는 초도 총비용으로 환산한 '초도 완전원가'라 양산 때보다 높게 나옵니다. 월 고정운영비에는 런칭 전 총액을 소진기간으로 나눈 월 상각이 포함됩니다 (계산기 결과는 이 시트의 판정과 근사치로만 같습니다).</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,7 @@
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>순매출 (VAT 제외 판매가)</t>
+          <t>판매 단위당 순매출 (VAT 제외 판매가)</t>
         </is>
       </c>
       <c r="B44" s="12">
@@ -1771,7 +1771,7 @@
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>고객 지불액 (VAT 포함)</t>
+          <t>판매 단위당 고객 지불액 (VAT 포함)</t>
         </is>
       </c>
       <c r="B45" s="12">
@@ -1964,7 +1964,7 @@
         </is>
       </c>
       <c r="B59" s="18">
-        <f>IF(NOT($B$43),"필수 입력(양산 수량·월 목표 판매량, 판매가, 초도 탭의 부가세율·VAT 여부)을 채워 주세요",IF(NOT(ISNUMBER($B$51)),"비용 입력을 확인하세요",IF($B$51&lt;=0,"판매 단위당 공헌이익이 0 이하입니다 — 팔수록 손해. 가격·원가·수수료를 다시 검토하세요",IF(NOT(ISNUMBER($B$56)),"고정비·수명주기 입력을 확인하세요",IF($B$56&gt;1,"목표 월 판매량으로는 본전이 안 됩니다 — 월 손익분기 "&amp;TEXT($B$55,"#,##0.#")&amp;"단위가 필요합니다","목표 월 판매량으로 본전 가능 — 월 "&amp;TEXT($B$55,"#,##0.#")&amp;"단위 이상 판매 필요")))))</f>
+        <f>IF(NOT($B$43),"필수 입력(양산 수량·월 목표 판매량, 판매가, 초도 탭의 부가세율·VAT 여부)을 채워 주세요",IF(NOT(ISNUMBER($B$51)),"비용 입력을 확인하세요",IF($B$51&lt;=0,"판매 단위당 공헌이익이 0 이하입니다 — 팔수록 손해. 가격·원가·수수료를 다시 검토하세요",IF(NOT(ISNUMBER($B$56)),"고정비·수명주기 입력을 확인하세요",IF($B$56&gt;1,"목표 월 판매량으로는 본전이 안 됩니다 — 월 손익분기 "&amp;IF(ROUND($B$55,1)=INT(ROUND($B$55,1)),TEXT(ROUND($B$55,1),"#,##0"),TEXT(ROUND($B$55,1),"#,##0.0"))&amp;"단위가 필요합니다","목표 월 판매량으로 본전 가능 — 월 "&amp;IF(ROUND($B$55,1)=INT(ROUND($B$55,1)),TEXT(ROUND($B$55,1),"#,##0"),TEXT(ROUND($B$55,1),"#,##0.0"))&amp;"단위 이상 판매 필요")))))</f>
         <v/>
       </c>
     </row>
@@ -1979,10 +1979,10 @@
       <c r="D61" s="4" t="n"/>
       <c r="E61" s="4" t="n"/>
     </row>
-    <row r="62" ht="15" customHeight="1">
+    <row r="62" ht="30" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>웹 계산기의 같은 이름 칸에 옮겨 적으세요 (양산 기준).</t>
+          <t>이 표(라벨과 값 두 열)를 복사해 웹 계산기의 '시트 값 붙여넣기'에 붙여넣으면 자동으로 채워집니다 (양산 기준). 직접 옮겨 적어도 됩니다.</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>판매가 (KRW)</t>
+          <t>판매 단위당 판매가 (KRW)</t>
         </is>
       </c>
       <c r="B6" s="12">
@@ -2190,7 +2190,7 @@
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>순매출 (VAT 제외)</t>
+          <t>판매 단위당 순매출 (VAT 제외)</t>
         </is>
       </c>
       <c r="B7" s="12">
@@ -2372,7 +2372,7 @@
         </is>
       </c>
       <c r="B16" s="18">
-        <f>IF(NOT(AND(ISNUMBER(B10),ISNUMBER(C10))),"두 탭의 필수 입력을 채우면 비교가 표시됩니다","양산하면 판매 단위당 직접원가가 "&amp;TEXT(ABS(C14),"0%")&amp;IF(C14&gt;=0," 낮아지고"," 높아지고")&amp;", 판매 단위당 공헌이익은 "&amp;TEXT(B10,"#,##0")&amp;"원에서 "&amp;TEXT(C10,"#,##0")&amp;"원이 됩니다. 월 손익분기는 "&amp;IF(AND(ISNUMBER(B12),ISNUMBER(C12)),TEXT(B12,"#,##0.#")&amp;"단위에서 "&amp;TEXT(C12,"#,##0.#")&amp;"단위로 바뀝니다.","확인이 필요합니다."))</f>
+        <f>IF(NOT(AND(ISNUMBER(B10),ISNUMBER(C10))),"두 탭의 필수 입력을 채우면 비교가 표시됩니다","양산하면 판매 단위당 직접원가가 "&amp;TEXT(ABS(C14),"0%")&amp;IF(C14&gt;=0," 낮아지고"," 높아지고")&amp;", 판매 단위당 공헌이익은 "&amp;TEXT(B10,"#,##0")&amp;"원에서 "&amp;TEXT(C10,"#,##0")&amp;"원이 됩니다. 월 손익분기는 "&amp;IF(AND(ISNUMBER(B12),ISNUMBER(C12)),IF(ROUND(B12,1)=INT(ROUND(B12,1)),TEXT(ROUND(B12,1),"#,##0"),TEXT(ROUND(B12,1),"#,##0.0"))&amp;"단위에서 "&amp;IF(ROUND(C12,1)=INT(ROUND(C12,1)),TEXT(ROUND(C12,1),"#,##0"),TEXT(ROUND(C12,1),"#,##0.0"))&amp;"단위로 바뀝니다.","확인이 필요합니다."))</f>
         <v/>
       </c>
     </row>
@@ -2436,14 +2436,14 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="192" customHeight="1">
+    <row r="6" ht="208" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
         <is>
           <t>① 1. 가정: 업종, 판매 단위(낱개 1개, 6개입 세트, 1건처럼 한 번 팔 때의 단위. 판매가·수량·모든 비용이 이 단위 기준입니다), 초도생산 수량(판매 단위 수. 서비스는 수용 한도가 아니라 이 기간 안에 팔려는 목표 판매 수), 목표 소진기간(서비스는 목표 판매 기간, 개월), 판매가, 부가세, VAT 포함 여부를 입력합니다.
 ② 2. 만드는 활동: 런칭 직전까지 만드는 데 드는 일(to-do)을 한 줄씩 적고 그 일에 드는 총비용을 적습니다. 구분은 필요 없습니다. 제조는 재료·가공·금형·장치·포장, 서비스는 기획·개발·디자인 인건비 등입니다.
 ③ 3. 파는 활동: 런칭 전에 쓰는 총비용은 '런칭 전 총액'으로, 팔 때마다 붙는 비용은 '판매 시 …'로 구분을 고릅니다. 구분을 고르지 않은 행은 합계에서 빠지며, 표 아래 '구분을 고르지 않은 행 수'가 0이 아니면 선택하라는 뜻입니다.
 ④ 3-2. 월 고정운영비: 물량과 무관하게 매달 나가는 비용을 적습니다.
-⑤ 4. 판정에서 본전 가능 여부를 읽고, 5. 계산기에 입력할 값을 웹 계산기에 옮겨 적습니다.</t>
+⑤ 4. 판정에서 본전 가능 여부를 읽고, 5. 계산기에 입력할 값 표(라벨과 값 두 열)를 복사해 웹 계산기의 '시트 값 붙여넣기'에 붙여넣습니다(직접 옮겨 적어도 됩니다).</t>
         </is>
       </c>
     </row>

</xml_diff>